<commit_message>
Added example: "Example5. Semantic with filter formulas"
</commit_message>
<xml_diff>
--- a/Parser/Example/InstructionExamples.xlsx
+++ b/Parser/Example/InstructionExamples.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MyFolder\Projects\ExcelToJsonUniversalParser\Repo\Parser2\Example\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MyFolder\Projects\TableToJsonUniversalParser\Repo\Parser\Example\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C28A760-D85F-4237-B56E-89F533DD5CB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63E9B106-4942-4A98-9421-6F87C8982255}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,17 +19,51 @@
     <sheet name="Lvl1" sheetId="7" r:id="rId4"/>
     <sheet name="Lvl2" sheetId="8" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Lvl2'!$M$53:$W$75</definedName>
+  </definedNames>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="646" uniqueCount="204">
   <si>
     <t>ignore</t>
   </si>
@@ -509,13 +543,145 @@
   </si>
   <si>
     <t>%wrap_amount_arg%</t>
+  </si>
+  <si>
+    <t>Example5. Semantic with filter formulas</t>
+  </si>
+  <si>
+    <t>season48</t>
+  </si>
+  <si>
+    <t>number</t>
+  </si>
+  <si>
+    <t>stages</t>
+  </si>
+  <si>
+    <t>season48stages</t>
+  </si>
+  <si>
+    <t>stage0</t>
+  </si>
+  <si>
+    <t>stage1</t>
+  </si>
+  <si>
+    <t>stage2</t>
+  </si>
+  <si>
+    <t>stage3</t>
+  </si>
+  <si>
+    <t>stage4</t>
+  </si>
+  <si>
+    <t>stage5</t>
+  </si>
+  <si>
+    <t>stage6</t>
+  </si>
+  <si>
+    <t>stage7</t>
+  </si>
+  <si>
+    <t>stage8</t>
+  </si>
+  <si>
+    <t>stage9</t>
+  </si>
+  <si>
+    <t>stage10</t>
+  </si>
+  <si>
+    <t>Titlte for stages number →</t>
+  </si>
+  <si>
+    <t>stageNumer</t>
+  </si>
+  <si>
+    <t>Common.GameplayConfigs.Player.Seasons.SeasonConfig+Stage</t>
+  </si>
+  <si>
+    <t>tokens</t>
+  </si>
+  <si>
+    <t>basicReward</t>
+  </si>
+  <si>
+    <t>SeasonLootBoxReward</t>
+  </si>
+  <si>
+    <t>LootBoxSilver</t>
+  </si>
+  <si>
+    <t>For parsing</t>
+  </si>
+  <si>
+    <t>passReward</t>
+  </si>
+  <si>
+    <t>LootBoxGold</t>
+  </si>
+  <si>
+    <t>stage</t>
+  </si>
+  <si>
+    <t>AliasFuncName</t>
+  </si>
+  <si>
+    <t>Tokens</t>
+  </si>
+  <si>
+    <t>isPremium</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Content</t>
+  </si>
+  <si>
+    <t>Count</t>
+  </si>
+  <si>
+    <t>LootBox</t>
+  </si>
+  <si>
+    <t>SeasonWheelTicketsReward</t>
+  </si>
+  <si>
+    <t>Basic</t>
+  </si>
+  <si>
+    <t>WheelTickets</t>
+  </si>
+  <si>
+    <t>SeasonCoreRandomBoosterReward</t>
+  </si>
+  <si>
+    <t>SeasonRandomBooster</t>
+  </si>
+  <si>
+    <t>RandBoosters</t>
+  </si>
+  <si>
+    <t>SeasonHardReward</t>
+  </si>
+  <si>
+    <t>HardCurrency</t>
+  </si>
+  <si>
+    <t>Premium</t>
+  </si>
+  <si>
+    <t>==IF(ROWS(FILTER($R$52:$R$73,($M$52:$M$73=$C49)*($N$52:$N$73=$J49)))=0,"",FILTER($R$52:$R$73,($M$52:$M$73=$C49)*($N$52:$N$73=$J49)))</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -542,8 +708,23 @@
       <family val="2"/>
       <charset val="204"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="204"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -562,8 +743,26 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF9BC2E6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCCCCCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFE599"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -571,29 +770,163 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -904,21 +1237,21 @@
       <c r="F1" t="s">
         <v>66</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="3" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="5" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" s="19" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="b">
         <v>1</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="19" t="s">
         <v>16</v>
       </c>
     </row>
@@ -1200,21 +1533,21 @@
       <c r="F1" t="s">
         <v>66</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="3" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="5" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" s="19" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="b">
         <v>1</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="19" t="s">
         <v>16</v>
       </c>
     </row>
@@ -1325,7 +1658,7 @@
     <col min="4" max="4" width="33.85546875" customWidth="1"/>
     <col min="5" max="5" width="12.85546875" customWidth="1"/>
     <col min="6" max="6" width="13.85546875" customWidth="1"/>
-    <col min="7" max="9" width="9.140625" style="4"/>
+    <col min="7" max="9" width="9.140625" style="3"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -1347,53 +1680,53 @@
       <c r="F1" t="s">
         <v>66</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="3" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="5" spans="1:12" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="b">
         <v>1</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5"/>
-      <c r="I5" s="5"/>
-      <c r="J5" s="5"/>
-      <c r="K5" s="5"/>
-      <c r="L5" s="5"/>
-    </row>
-    <row r="7" spans="1:12" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C5" s="19"/>
+      <c r="D5" s="19"/>
+      <c r="E5" s="19"/>
+      <c r="F5" s="19"/>
+      <c r="G5" s="19"/>
+      <c r="H5" s="19"/>
+      <c r="I5" s="19"/>
+      <c r="J5" s="19"/>
+      <c r="K5" s="19"/>
+      <c r="L5" s="19"/>
+    </row>
+    <row r="7" spans="1:12" collapsed="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="6"/>
-      <c r="D7" s="6"/>
-      <c r="E7" s="6"/>
-      <c r="F7" s="6"/>
-      <c r="G7" s="6"/>
-      <c r="H7" s="6"/>
-      <c r="I7" s="6"/>
-      <c r="J7" s="6"/>
-      <c r="K7" s="6"/>
-      <c r="L7" s="6"/>
-    </row>
-    <row r="8" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="C7" s="23"/>
+      <c r="D7" s="23"/>
+      <c r="E7" s="23"/>
+      <c r="F7" s="23"/>
+      <c r="G7" s="23"/>
+      <c r="H7" s="23"/>
+      <c r="I7" s="23"/>
+      <c r="J7" s="23"/>
+      <c r="K7" s="23"/>
+      <c r="L7" s="23"/>
+    </row>
+    <row r="8" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>7</v>
       </c>
@@ -1407,7 +1740,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="C9" t="s">
         <v>9</v>
       </c>
@@ -1418,7 +1751,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="C10" t="s">
         <v>11</v>
       </c>
@@ -1429,7 +1762,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="11" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="C11" t="s">
         <v>12</v>
       </c>
@@ -1440,26 +1773,26 @@
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25"/>
-    <row r="14" spans="1:12" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="14" spans="1:12" collapsed="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="B14" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="C14" s="6"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="6"/>
-      <c r="F14" s="6"/>
-      <c r="G14" s="6"/>
-      <c r="H14" s="6"/>
-      <c r="I14" s="6"/>
-      <c r="J14" s="6"/>
-      <c r="K14" s="6"/>
-      <c r="L14" s="6"/>
-    </row>
-    <row r="15" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="C14" s="23"/>
+      <c r="D14" s="23"/>
+      <c r="E14" s="23"/>
+      <c r="F14" s="23"/>
+      <c r="G14" s="23"/>
+      <c r="H14" s="23"/>
+      <c r="I14" s="23"/>
+      <c r="J14" s="23"/>
+      <c r="K14" s="23"/>
+      <c r="L14" s="23"/>
+    </row>
+    <row r="15" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>21</v>
       </c>
@@ -1473,7 +1806,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="16" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="C16" t="s">
         <v>24</v>
       </c>
@@ -1484,7 +1817,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="17" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="C17" t="s">
         <v>25</v>
       </c>
@@ -1495,7 +1828,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="C18" t="s">
         <v>27</v>
       </c>
@@ -1503,7 +1836,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="19" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="C19" t="s">
         <v>28</v>
       </c>
@@ -1514,7 +1847,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="20" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="C20" t="s">
         <v>29</v>
       </c>
@@ -1525,7 +1858,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="21" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="C21" t="s">
         <v>42</v>
       </c>
@@ -1536,45 +1869,45 @@
         <v>43</v>
       </c>
     </row>
-    <row r="22" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25"/>
-    <row r="24" spans="1:12" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="24" spans="1:12" collapsed="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="B24" s="6" t="s">
+      <c r="B24" s="23" t="s">
         <v>60</v>
       </c>
-      <c r="C24" s="6"/>
-      <c r="D24" s="6"/>
-      <c r="E24" s="6"/>
-      <c r="F24" s="6"/>
-      <c r="G24" s="6"/>
-      <c r="H24" s="6"/>
-      <c r="I24" s="6"/>
-      <c r="J24" s="6"/>
-      <c r="K24" s="6"/>
-      <c r="L24" s="6"/>
-    </row>
-    <row r="25" spans="1:12" s="9" customFormat="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="C24" s="23"/>
+      <c r="D24" s="23"/>
+      <c r="E24" s="23"/>
+      <c r="F24" s="23"/>
+      <c r="G24" s="23"/>
+      <c r="H24" s="23"/>
+      <c r="I24" s="23"/>
+      <c r="J24" s="23"/>
+      <c r="K24" s="23"/>
+      <c r="L24" s="23"/>
+    </row>
+    <row r="25" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="B25" s="6" t="s">
+      <c r="B25" s="23" t="s">
         <v>49</v>
       </c>
-      <c r="C25" s="6"/>
-      <c r="D25" s="6"/>
-      <c r="E25" s="6"/>
-      <c r="F25" s="6"/>
-      <c r="G25" s="6"/>
-      <c r="H25" s="6"/>
-      <c r="I25" s="6"/>
-      <c r="J25" s="6"/>
-      <c r="K25" s="6"/>
-      <c r="L25" s="6"/>
-    </row>
-    <row r="26" spans="1:12" outlineLevel="2" x14ac:dyDescent="0.25"/>
-    <row r="27" spans="1:12" outlineLevel="2" x14ac:dyDescent="0.25">
+      <c r="C25" s="23"/>
+      <c r="D25" s="23"/>
+      <c r="E25" s="23"/>
+      <c r="F25" s="23"/>
+      <c r="G25" s="23"/>
+      <c r="H25" s="23"/>
+      <c r="I25" s="23"/>
+      <c r="J25" s="23"/>
+      <c r="K25" s="23"/>
+      <c r="L25" s="23"/>
+    </row>
+    <row r="26" spans="1:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25"/>
+    <row r="27" spans="1:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
         <v>48</v>
       </c>
@@ -1588,7 +1921,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="28" spans="1:12" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="C28" t="s">
         <v>51</v>
       </c>
@@ -1599,7 +1932,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="29" spans="1:12" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="C29" t="s">
         <v>52</v>
       </c>
@@ -1610,28 +1943,28 @@
         <v>55</v>
       </c>
     </row>
-    <row r="30" spans="1:12" outlineLevel="2" x14ac:dyDescent="0.25"/>
-    <row r="31" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25"/>
-    <row r="32" spans="1:12" s="9" customFormat="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25"/>
+    <row r="31" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="32" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="B32" s="6" t="s">
+      <c r="B32" s="23" t="s">
         <v>62</v>
       </c>
-      <c r="C32" s="6"/>
-      <c r="D32" s="6"/>
-      <c r="E32" s="6"/>
-      <c r="F32" s="6"/>
-      <c r="G32" s="6"/>
-      <c r="H32" s="6"/>
-      <c r="I32" s="6"/>
-      <c r="J32" s="6"/>
-      <c r="K32" s="6"/>
-      <c r="L32" s="6"/>
-    </row>
-    <row r="33" spans="1:12" outlineLevel="2" x14ac:dyDescent="0.25"/>
-    <row r="34" spans="1:12" outlineLevel="2" x14ac:dyDescent="0.25">
+      <c r="C32" s="23"/>
+      <c r="D32" s="23"/>
+      <c r="E32" s="23"/>
+      <c r="F32" s="23"/>
+      <c r="G32" s="23"/>
+      <c r="H32" s="23"/>
+      <c r="I32" s="23"/>
+      <c r="J32" s="23"/>
+      <c r="K32" s="23"/>
+      <c r="L32" s="23"/>
+    </row>
+    <row r="33" spans="1:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25"/>
+    <row r="34" spans="1:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="B34" t="s">
         <v>63</v>
       </c>
@@ -1648,7 +1981,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="35" spans="1:12" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="C35" t="s">
         <v>51</v>
       </c>
@@ -1662,7 +1995,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="36" spans="1:12" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="C36" t="s">
         <v>52</v>
       </c>
@@ -1673,28 +2006,28 @@
         <v>67</v>
       </c>
     </row>
-    <row r="37" spans="1:12" outlineLevel="2" x14ac:dyDescent="0.25"/>
-    <row r="38" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25"/>
-    <row r="39" spans="1:12" s="9" customFormat="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25"/>
+    <row r="38" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="39" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="B39" s="6" t="s">
+      <c r="B39" s="23" t="s">
         <v>69</v>
       </c>
-      <c r="C39" s="6"/>
-      <c r="D39" s="6"/>
-      <c r="E39" s="6"/>
-      <c r="F39" s="6"/>
-      <c r="G39" s="6"/>
-      <c r="H39" s="6"/>
-      <c r="I39" s="6"/>
-      <c r="J39" s="6"/>
-      <c r="K39" s="6"/>
-      <c r="L39" s="6"/>
-    </row>
-    <row r="40" spans="1:12" outlineLevel="2" x14ac:dyDescent="0.25"/>
-    <row r="41" spans="1:12" outlineLevel="2" x14ac:dyDescent="0.25">
+      <c r="C39" s="23"/>
+      <c r="D39" s="23"/>
+      <c r="E39" s="23"/>
+      <c r="F39" s="23"/>
+      <c r="G39" s="23"/>
+      <c r="H39" s="23"/>
+      <c r="I39" s="23"/>
+      <c r="J39" s="23"/>
+      <c r="K39" s="23"/>
+      <c r="L39" s="23"/>
+    </row>
+    <row r="40" spans="1:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25"/>
+    <row r="41" spans="1:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="B41" t="s">
         <v>73</v>
       </c>
@@ -1711,7 +2044,7 @@
         <v>1500</v>
       </c>
     </row>
-    <row r="42" spans="1:12" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="C42" t="s">
         <v>71</v>
       </c>
@@ -1725,27 +2058,27 @@
         <v>1500</v>
       </c>
     </row>
-    <row r="43" spans="1:12" outlineLevel="2" x14ac:dyDescent="0.25"/>
-    <row r="44" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25"/>
-    <row r="45" spans="1:12" s="9" customFormat="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25"/>
+    <row r="44" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="45" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="B45" s="6" t="s">
+      <c r="B45" s="23" t="s">
         <v>94</v>
       </c>
-      <c r="C45" s="6"/>
-      <c r="D45" s="6"/>
-      <c r="E45" s="6"/>
-      <c r="F45" s="6"/>
-      <c r="G45" s="6"/>
-      <c r="H45" s="6"/>
-      <c r="I45" s="6"/>
-      <c r="J45" s="6"/>
-      <c r="K45" s="6"/>
-      <c r="L45" s="6"/>
-    </row>
-    <row r="46" spans="1:12" outlineLevel="2" x14ac:dyDescent="0.25">
+      <c r="C45" s="23"/>
+      <c r="D45" s="23"/>
+      <c r="E45" s="23"/>
+      <c r="F45" s="23"/>
+      <c r="G45" s="23"/>
+      <c r="H45" s="23"/>
+      <c r="I45" s="23"/>
+      <c r="J45" s="23"/>
+      <c r="K45" s="23"/>
+      <c r="L45" s="23"/>
+    </row>
+    <row r="46" spans="1:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="B46" t="s">
         <v>91</v>
       </c>
@@ -1762,27 +2095,27 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="47" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25"/>
-    <row r="48" spans="1:12" s="9" customFormat="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="48" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="B48" s="6" t="s">
+      <c r="B48" s="23" t="s">
         <v>74</v>
       </c>
-      <c r="C48" s="6"/>
-      <c r="D48" s="6"/>
-      <c r="E48" s="6"/>
-      <c r="F48" s="6"/>
-      <c r="G48" s="6"/>
-      <c r="H48" s="6"/>
-      <c r="I48" s="6"/>
-      <c r="J48" s="6"/>
-      <c r="K48" s="6"/>
-      <c r="L48" s="6"/>
-    </row>
-    <row r="49" spans="1:12" outlineLevel="2" x14ac:dyDescent="0.25"/>
-    <row r="50" spans="1:12" outlineLevel="2" x14ac:dyDescent="0.25">
+      <c r="C48" s="23"/>
+      <c r="D48" s="23"/>
+      <c r="E48" s="23"/>
+      <c r="F48" s="23"/>
+      <c r="G48" s="23"/>
+      <c r="H48" s="23"/>
+      <c r="I48" s="23"/>
+      <c r="J48" s="23"/>
+      <c r="K48" s="23"/>
+      <c r="L48" s="23"/>
+    </row>
+    <row r="49" spans="1:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25"/>
+    <row r="50" spans="1:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="B50" t="s">
         <v>84</v>
       </c>
@@ -1792,34 +2125,34 @@
       <c r="D50" t="s">
         <v>85</v>
       </c>
-      <c r="G50" s="4">
+      <c r="G50" s="3">
         <v>200</v>
       </c>
-      <c r="H50" s="4" t="s">
+      <c r="H50" s="3" t="s">
         <v>23</v>
       </c>
       <c r="I50" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:12" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="C51" t="s">
         <v>87</v>
       </c>
       <c r="D51" t="s">
         <v>88</v>
       </c>
-      <c r="G51" s="4">
+      <c r="G51" s="3">
         <v>200</v>
       </c>
-      <c r="H51" s="4" t="s">
+      <c r="H51" s="3" t="s">
         <v>23</v>
       </c>
       <c r="I51" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="1:12" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="C52" t="s">
         <v>90</v>
       </c>
@@ -1832,35 +2165,35 @@
       <c r="F52">
         <v>1500</v>
       </c>
-      <c r="H52" s="4" t="s">
+      <c r="H52" s="3" t="s">
         <v>23</v>
       </c>
       <c r="I52" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:12" outlineLevel="2" x14ac:dyDescent="0.25"/>
-    <row r="54" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25"/>
-    <row r="56" spans="1:12" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25"/>
+    <row r="54" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="56" spans="1:12" collapsed="1" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="B56" s="6" t="s">
+      <c r="B56" s="23" t="s">
         <v>95</v>
       </c>
-      <c r="C56" s="6"/>
-      <c r="D56" s="6"/>
-      <c r="E56" s="6"/>
-      <c r="F56" s="6"/>
-      <c r="G56" s="6"/>
-      <c r="H56" s="6"/>
-      <c r="I56" s="6"/>
-      <c r="J56" s="6"/>
-      <c r="K56" s="6"/>
-      <c r="L56" s="6"/>
-    </row>
-    <row r="57" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25"/>
-    <row r="58" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="C56" s="23"/>
+      <c r="D56" s="23"/>
+      <c r="E56" s="23"/>
+      <c r="F56" s="23"/>
+      <c r="G56" s="23"/>
+      <c r="H56" s="23"/>
+      <c r="I56" s="23"/>
+      <c r="J56" s="23"/>
+      <c r="K56" s="23"/>
+      <c r="L56" s="23"/>
+    </row>
+    <row r="57" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="58" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A58" t="b">
         <v>1</v>
       </c>
@@ -1871,7 +2204,7 @@
       <c r="H58"/>
       <c r="I58"/>
     </row>
-    <row r="59" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A59" t="b">
         <v>1</v>
       </c>
@@ -1882,7 +2215,7 @@
       <c r="H59"/>
       <c r="I59"/>
     </row>
-    <row r="60" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A60" t="b">
         <v>0</v>
       </c>
@@ -1902,7 +2235,7 @@
       <c r="H60"/>
       <c r="I60"/>
     </row>
-    <row r="61" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="C61" t="s">
         <v>100</v>
       </c>
@@ -1916,7 +2249,7 @@
       <c r="H61"/>
       <c r="I61"/>
     </row>
-    <row r="62" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="C62" t="s">
         <v>101</v>
       </c>
@@ -1927,7 +2260,7 @@
       <c r="H62"/>
       <c r="I62"/>
     </row>
-    <row r="63" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="C63" t="s">
         <v>79</v>
       </c>
@@ -1941,7 +2274,7 @@
       <c r="H63"/>
       <c r="I63"/>
     </row>
-    <row r="64" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="C64" t="s">
         <v>80</v>
       </c>
@@ -1955,7 +2288,7 @@
       <c r="H64"/>
       <c r="I64"/>
     </row>
-    <row r="65" spans="3:6" customFormat="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="3:6" customFormat="1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="C65" t="s">
         <v>104</v>
       </c>
@@ -1966,7 +2299,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="66" spans="3:6" customFormat="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="3:6" customFormat="1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="C66" t="s">
         <v>106</v>
       </c>
@@ -1977,7 +2310,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="67" spans="3:6" customFormat="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="3:6" customFormat="1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="C67" t="s">
         <v>106</v>
       </c>
@@ -1988,7 +2321,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="68" spans="3:6" customFormat="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="3:6" customFormat="1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="C68" t="s">
         <v>109</v>
       </c>
@@ -1999,7 +2332,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="69" spans="3:6" customFormat="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="3:6" customFormat="1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="C69" t="s">
         <v>111</v>
       </c>
@@ -2010,7 +2343,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="70" spans="3:6" customFormat="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="3:6" customFormat="1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="C70" t="s">
         <v>113</v>
       </c>
@@ -2021,7 +2354,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="71" spans="3:6" customFormat="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="3:6" customFormat="1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="C71" t="s">
         <v>115</v>
       </c>
@@ -2035,8 +2368,8 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="72" spans="3:6" customFormat="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
-    <row r="73" spans="3:6" customFormat="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="3:6" customFormat="1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="73" spans="3:6" customFormat="1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="C73" t="s">
         <v>116</v>
       </c>
@@ -2050,7 +2383,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="74" spans="3:6" customFormat="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="3:6" customFormat="1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="E74" t="s">
         <v>82</v>
       </c>
@@ -2058,7 +2391,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="75" spans="3:6" customFormat="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="3:6" customFormat="1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="C75" t="s">
         <v>118</v>
       </c>
@@ -2072,7 +2405,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="76" spans="3:6" customFormat="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="3:6" customFormat="1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="C76" t="s">
         <v>119</v>
       </c>
@@ -2086,7 +2419,7 @@
         <v>1234</v>
       </c>
     </row>
-    <row r="77" spans="3:6" customFormat="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="3:6" customFormat="1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="E77" t="s">
         <v>58</v>
       </c>
@@ -2094,7 +2427,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="78" spans="3:6" customFormat="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="3:6" customFormat="1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="C78" t="s">
         <v>121</v>
       </c>
@@ -2105,8 +2438,8 @@
         <v>122</v>
       </c>
     </row>
-    <row r="79" spans="3:6" customFormat="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
-    <row r="80" spans="3:6" customFormat="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="3:6" customFormat="1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="80" spans="3:6" customFormat="1" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="C80" t="s">
         <v>123</v>
       </c>
@@ -2114,12 +2447,12 @@
         <v>124</v>
       </c>
     </row>
-    <row r="81" spans="1:9" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="G81"/>
       <c r="H81"/>
       <c r="I81"/>
     </row>
-    <row r="82" spans="1:9" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="C82" t="s">
         <v>125</v>
       </c>
@@ -2136,12 +2469,12 @@
       <c r="H82"/>
       <c r="I82"/>
     </row>
-    <row r="83" spans="1:9" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="G83"/>
       <c r="H83"/>
       <c r="I83"/>
     </row>
-    <row r="84" spans="1:9" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="C84" t="s">
         <v>128</v>
       </c>
@@ -2158,7 +2491,7 @@
       <c r="H84"/>
       <c r="I84"/>
     </row>
-    <row r="85" spans="1:9" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="C85" t="s">
         <v>130</v>
       </c>
@@ -2175,12 +2508,12 @@
       <c r="H85"/>
       <c r="I85"/>
     </row>
-    <row r="86" spans="1:9" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="G86"/>
       <c r="H86"/>
       <c r="I86"/>
     </row>
-    <row r="87" spans="1:9" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="C87" t="s">
         <v>133</v>
       </c>
@@ -2197,7 +2530,7 @@
         <v>54321</v>
       </c>
     </row>
-    <row r="88" spans="1:9" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="C88" t="s">
         <v>135</v>
       </c>
@@ -2214,12 +2547,12 @@
         <v>98765</v>
       </c>
     </row>
-    <row r="89" spans="1:9" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="G89"/>
       <c r="H89"/>
       <c r="I89"/>
     </row>
-    <row r="90" spans="1:9" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A90" t="b">
         <v>0</v>
       </c>
@@ -2227,7 +2560,7 @@
       <c r="H90"/>
       <c r="I90"/>
     </row>
-    <row r="91" spans="1:9" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A91" t="b">
         <v>0</v>
       </c>
@@ -2247,65 +2580,112 @@
       <c r="H91"/>
       <c r="I91"/>
     </row>
-    <row r="92" spans="1:9" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="F92" s="4"/>
+    <row r="92" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="F92" s="3"/>
       <c r="I92"/>
     </row>
-    <row r="93" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="F93" s="4"/>
+    <row r="93" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F93" s="3"/>
       <c r="I93"/>
     </row>
-    <row r="94" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="F94" s="4"/>
-      <c r="I94"/>
-    </row>
-    <row r="95" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="F95" s="4"/>
+    <row r="94" spans="1:12" ht="15.75" collapsed="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A94" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B94" s="20" t="s">
+        <v>160</v>
+      </c>
+      <c r="C94" s="21"/>
+      <c r="D94" s="21"/>
+      <c r="E94" s="21"/>
+      <c r="F94" s="21"/>
+      <c r="G94" s="21"/>
+      <c r="H94" s="21"/>
+      <c r="I94" s="21"/>
+      <c r="J94" s="21"/>
+      <c r="K94" s="21"/>
+      <c r="L94" s="22"/>
+    </row>
+    <row r="95" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="F95" s="3"/>
       <c r="I95"/>
     </row>
-    <row r="96" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="F96" s="4"/>
+    <row r="96" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B96" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="C96" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="D96" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="E96" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="F96" s="3"/>
       <c r="I96"/>
     </row>
-    <row r="97" spans="6:9" x14ac:dyDescent="0.25">
-      <c r="F97" s="4"/>
+    <row r="97" spans="2:9" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B97" s="5"/>
+      <c r="C97" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="D97" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="E97" s="9">
+        <v>48</v>
+      </c>
+      <c r="F97" s="3"/>
       <c r="I97"/>
     </row>
-    <row r="98" spans="6:9" x14ac:dyDescent="0.25">
-      <c r="F98" s="4"/>
+    <row r="98" spans="2:9" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B98" s="5"/>
+      <c r="C98" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="D98" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="E98" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="F98" s="3"/>
       <c r="I98"/>
     </row>
-    <row r="99" spans="6:9" x14ac:dyDescent="0.25">
-      <c r="F99" s="4"/>
+    <row r="99" spans="2:9" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="F99" s="3"/>
       <c r="I99"/>
     </row>
-    <row r="100" spans="6:9" x14ac:dyDescent="0.25">
-      <c r="F100" s="4"/>
+    <row r="100" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="F100" s="3"/>
       <c r="I100"/>
     </row>
-    <row r="101" spans="6:9" x14ac:dyDescent="0.25">
-      <c r="F101" s="4"/>
+    <row r="101" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="F101" s="3"/>
       <c r="I101"/>
     </row>
-    <row r="102" spans="6:9" x14ac:dyDescent="0.25">
-      <c r="F102" s="4"/>
+    <row r="102" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="F102" s="3"/>
       <c r="I102"/>
     </row>
-    <row r="103" spans="6:9" x14ac:dyDescent="0.25">
-      <c r="F103" s="4"/>
+    <row r="103" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="F103" s="3"/>
       <c r="I103"/>
     </row>
-    <row r="104" spans="6:9" x14ac:dyDescent="0.25">
-      <c r="F104" s="4"/>
+    <row r="104" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="F104" s="3"/>
       <c r="I104"/>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="11">
     <mergeCell ref="B5:L5"/>
     <mergeCell ref="B7:L7"/>
     <mergeCell ref="B14:L14"/>
     <mergeCell ref="B24:L24"/>
     <mergeCell ref="B32:L32"/>
+    <mergeCell ref="B94:L94"/>
     <mergeCell ref="B39:L39"/>
     <mergeCell ref="B45:L45"/>
     <mergeCell ref="B25:L25"/>
@@ -2323,577 +2703,710 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:L69"/>
+  <dimension ref="A1:L84"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.85546875" style="8" customWidth="1"/>
-    <col min="2" max="2" width="25" style="8" customWidth="1"/>
-    <col min="3" max="3" width="12.7109375" style="8" customWidth="1"/>
-    <col min="4" max="4" width="19.42578125" style="8" customWidth="1"/>
-    <col min="5" max="5" width="34.5703125" style="8" customWidth="1"/>
-    <col min="6" max="6" width="17.28515625" style="8" customWidth="1"/>
-    <col min="7" max="16384" width="9.140625" style="8"/>
+    <col min="1" max="1" width="15.85546875" customWidth="1"/>
+    <col min="2" max="2" width="25" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" customWidth="1"/>
+    <col min="4" max="4" width="19.42578125" customWidth="1"/>
+    <col min="5" max="5" width="34.5703125" customWidth="1"/>
+    <col min="6" max="6" width="17.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="8" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="8" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="8" t="s">
+      <c r="F1" t="s">
         <v>66</v>
       </c>
-      <c r="G1" s="8" t="s">
+      <c r="G1" t="s">
         <v>81</v>
       </c>
-      <c r="H1" s="8" t="s">
+      <c r="H1" t="s">
         <v>82</v>
       </c>
-      <c r="I1" s="8" t="s">
+      <c r="I1" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="5" spans="1:12" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="b">
         <v>1</v>
       </c>
-      <c r="B5" s="5" t="str">
+      <c r="B5" s="19" t="str">
         <f>Lvl0!B5</f>
         <v>This row start parsing</v>
       </c>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5"/>
-      <c r="I5" s="5"/>
-      <c r="J5" s="5"/>
-      <c r="K5" s="5"/>
-      <c r="L5" s="5"/>
-    </row>
-    <row r="7" spans="1:12" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C5" s="19"/>
+      <c r="D5" s="19"/>
+      <c r="E5" s="19"/>
+      <c r="F5" s="19"/>
+      <c r="G5" s="19"/>
+      <c r="H5" s="19"/>
+      <c r="I5" s="19"/>
+      <c r="J5" s="19"/>
+      <c r="K5" s="19"/>
+      <c r="L5" s="19"/>
+    </row>
+    <row r="7" spans="1:12" collapsed="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="B7" s="6" t="str">
+      <c r="B7" s="23" t="str">
         <f>Lvl0!B7</f>
         <v>Example1. Parsing target json</v>
       </c>
-      <c r="C7" s="6"/>
-      <c r="D7" s="6"/>
-      <c r="E7" s="6"/>
-      <c r="F7" s="6"/>
-      <c r="G7" s="6"/>
-      <c r="H7" s="6"/>
-      <c r="I7" s="6"/>
-      <c r="J7" s="6"/>
-      <c r="K7" s="6"/>
-      <c r="L7" s="6"/>
-    </row>
-    <row r="8" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="8" t="s">
+      <c r="C7" s="23"/>
+      <c r="D7" s="23"/>
+      <c r="E7" s="23"/>
+      <c r="F7" s="23"/>
+      <c r="G7" s="23"/>
+      <c r="H7" s="23"/>
+      <c r="I7" s="23"/>
+      <c r="J7" s="23"/>
+      <c r="K7" s="23"/>
+      <c r="L7" s="23"/>
+    </row>
+    <row r="8" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
         <v>14</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" t="s">
         <v>5</v>
       </c>
-      <c r="E8" s="8" t="s">
+      <c r="E8" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="C9" s="8" t="s">
+    <row r="9" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="C9" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="D9" t="s">
         <v>5</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="E9" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25"/>
-    <row r="12" spans="1:12" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="12" spans="1:12" collapsed="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="B12" s="6" t="str">
+      <c r="B12" s="23" t="str">
         <f>Lvl0!B14</f>
         <v>Example2. Types variation</v>
       </c>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="6"/>
-      <c r="H12" s="6"/>
-      <c r="I12" s="6"/>
-      <c r="J12" s="6"/>
-      <c r="K12" s="6"/>
-      <c r="L12" s="6"/>
-    </row>
-    <row r="13" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="8" t="s">
+      <c r="C12" s="23"/>
+      <c r="D12" s="23"/>
+      <c r="E12" s="23"/>
+      <c r="F12" s="23"/>
+      <c r="G12" s="23"/>
+      <c r="H12" s="23"/>
+      <c r="I12" s="23"/>
+      <c r="J12" s="23"/>
+      <c r="K12" s="23"/>
+      <c r="L12" s="23"/>
+    </row>
+    <row r="13" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
         <v>32</v>
       </c>
-      <c r="C13" s="8" t="s">
+      <c r="C13" t="s">
         <v>34</v>
       </c>
-      <c r="D13" s="8" t="s">
+      <c r="D13" t="s">
         <v>5</v>
       </c>
-      <c r="E13" s="8" t="s">
+      <c r="E13" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="14" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="C14" s="8" t="s">
+    <row r="14" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="C14" t="s">
         <v>35</v>
       </c>
-      <c r="D14" s="8" t="s">
+      <c r="D14" t="s">
         <v>6</v>
       </c>
-      <c r="E14" s="8">
+      <c r="E14">
         <v>12345</v>
       </c>
     </row>
-    <row r="15" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25"/>
-    <row r="16" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="8" t="s">
+    <row r="15" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="16" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B16" t="s">
         <v>31</v>
       </c>
-      <c r="D16" s="8" t="s">
+      <c r="D16" t="s">
         <v>5</v>
       </c>
-      <c r="E16" s="8" t="s">
+      <c r="E16" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="17" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="D17" s="8" t="s">
+    <row r="17" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="D17" t="s">
         <v>5</v>
       </c>
-      <c r="E17" s="8" t="s">
+      <c r="E17" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="18" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="D18" s="8" t="s">
+    <row r="18" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="D18" t="s">
         <v>5</v>
       </c>
-      <c r="E18" s="8" t="s">
+      <c r="E18" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="19" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="D19" s="8" t="s">
+    <row r="19" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="D19" t="s">
         <v>5</v>
       </c>
-      <c r="E19" s="8" t="s">
+      <c r="E19" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="20" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="D20" s="8" t="s">
+    <row r="20" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="D20" t="s">
         <v>5</v>
       </c>
-      <c r="E20" s="8" t="s">
+      <c r="E20" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="21" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="8" t="s">
+    <row r="21" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B21" t="s">
         <v>43</v>
       </c>
-      <c r="D21" s="8" t="s">
+      <c r="D21" t="s">
         <v>13</v>
       </c>
-      <c r="E21" s="8" t="s">
+      <c r="E21" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="22" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="D22" s="8" t="s">
+    <row r="22" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="D22" t="s">
         <v>13</v>
       </c>
-      <c r="E22" s="8" t="s">
+      <c r="E22" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="23" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="D23" s="8" t="s">
+    <row r="23" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="D23" t="s">
         <v>13</v>
       </c>
-      <c r="E23" s="8" t="s">
+      <c r="E23" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="24" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25"/>
-    <row r="26" spans="1:12" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="26" spans="1:12" collapsed="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="B26" s="6" t="str">
+      <c r="B26" s="23" t="str">
         <f>Lvl0!B24</f>
         <v>Example3 Alias function</v>
       </c>
-      <c r="C26" s="6"/>
-      <c r="D26" s="6"/>
-      <c r="E26" s="6"/>
-      <c r="F26" s="6"/>
-      <c r="G26" s="6"/>
-      <c r="H26" s="6"/>
-      <c r="I26" s="6"/>
-      <c r="J26" s="6"/>
-      <c r="K26" s="6"/>
-      <c r="L26" s="6"/>
-    </row>
-    <row r="27" spans="1:12" s="9" customFormat="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="C26" s="23"/>
+      <c r="D26" s="23"/>
+      <c r="E26" s="23"/>
+      <c r="F26" s="23"/>
+      <c r="G26" s="23"/>
+      <c r="H26" s="23"/>
+      <c r="I26" s="23"/>
+      <c r="J26" s="23"/>
+      <c r="K26" s="23"/>
+      <c r="L26" s="23"/>
+    </row>
+    <row r="27" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="B27" s="6" t="str">
+      <c r="B27" s="23" t="str">
         <f>Lvl0!B25</f>
         <v>Example3.1 Alias function. Semantics without alias func</v>
       </c>
-      <c r="C27" s="6"/>
-      <c r="D27" s="6"/>
-      <c r="E27" s="6"/>
-      <c r="F27" s="6"/>
-      <c r="G27" s="6"/>
-      <c r="H27" s="6"/>
-      <c r="I27" s="6"/>
-      <c r="J27" s="6"/>
-      <c r="K27" s="6"/>
-      <c r="L27" s="6"/>
-    </row>
-    <row r="28" spans="1:12" outlineLevel="2" x14ac:dyDescent="0.25"/>
-    <row r="29" spans="1:12" outlineLevel="2" x14ac:dyDescent="0.25">
-      <c r="B29" s="8" t="s">
+      <c r="C27" s="23"/>
+      <c r="D27" s="23"/>
+      <c r="E27" s="23"/>
+      <c r="F27" s="23"/>
+      <c r="G27" s="23"/>
+      <c r="H27" s="23"/>
+      <c r="I27" s="23"/>
+      <c r="J27" s="23"/>
+      <c r="K27" s="23"/>
+      <c r="L27" s="23"/>
+    </row>
+    <row r="28" spans="1:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25"/>
+    <row r="29" spans="1:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
+      <c r="B29" t="s">
         <v>53</v>
       </c>
-      <c r="C29" s="8" t="s">
+      <c r="C29" t="s">
         <v>56</v>
       </c>
-      <c r="D29" s="8" t="s">
+      <c r="D29" t="s">
         <v>5</v>
       </c>
-      <c r="E29" s="8" t="s">
+      <c r="E29" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="30" spans="1:12" outlineLevel="2" x14ac:dyDescent="0.25">
-      <c r="C30" s="8" t="s">
+    <row r="30" spans="1:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
+      <c r="C30" t="s">
         <v>58</v>
       </c>
-      <c r="D30" s="8" t="s">
+      <c r="D30" t="s">
         <v>6</v>
       </c>
-      <c r="E30" s="8">
+      <c r="E30">
         <v>100</v>
       </c>
     </row>
-    <row r="31" spans="1:12" outlineLevel="2" x14ac:dyDescent="0.25">
-      <c r="B31" s="8" t="s">
+    <row r="31" spans="1:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
+      <c r="B31" t="s">
         <v>54</v>
       </c>
-      <c r="C31" s="8" t="s">
+      <c r="C31" t="s">
         <v>56</v>
       </c>
-      <c r="D31" s="8" t="s">
+      <c r="D31" t="s">
         <v>5</v>
       </c>
-      <c r="E31" s="8" t="s">
+      <c r="E31" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="32" spans="1:12" outlineLevel="2" x14ac:dyDescent="0.25">
-      <c r="C32" s="8" t="s">
+    <row r="32" spans="1:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
+      <c r="C32" t="s">
         <v>58</v>
       </c>
-      <c r="D32" s="8" t="s">
+      <c r="D32" t="s">
         <v>6</v>
       </c>
-      <c r="E32" s="8">
+      <c r="E32">
         <v>350</v>
       </c>
     </row>
-    <row r="33" spans="1:12" outlineLevel="2" x14ac:dyDescent="0.25">
-      <c r="B33" s="8" t="s">
+    <row r="33" spans="1:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
+      <c r="B33" t="s">
         <v>55</v>
       </c>
-      <c r="D33" s="8" t="s">
+      <c r="D33" t="s">
         <v>13</v>
       </c>
-      <c r="E33" s="8" t="s">
+      <c r="E33" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="34" spans="1:12" outlineLevel="2" x14ac:dyDescent="0.25">
-      <c r="D34" s="8" t="s">
+    <row r="34" spans="1:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
+      <c r="D34" t="s">
         <v>13</v>
       </c>
-      <c r="E34" s="8" t="s">
+      <c r="E34" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="35" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25"/>
-    <row r="36" spans="1:12" s="9" customFormat="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="36" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="B36" s="6" t="str">
+      <c r="B36" s="23" t="str">
         <f>Lvl0!B32</f>
         <v>Example3.2 Alias function. Semantics with alias func</v>
       </c>
-      <c r="C36" s="6"/>
-      <c r="D36" s="6"/>
-      <c r="E36" s="6"/>
-      <c r="F36" s="6"/>
-      <c r="G36" s="6"/>
-      <c r="H36" s="6"/>
-      <c r="I36" s="6"/>
-      <c r="J36" s="6"/>
-      <c r="K36" s="6"/>
-      <c r="L36" s="6"/>
-    </row>
-    <row r="37" spans="1:12" outlineLevel="2" x14ac:dyDescent="0.25">
-      <c r="B37" s="8" t="s">
+      <c r="C36" s="23"/>
+      <c r="D36" s="23"/>
+      <c r="E36" s="23"/>
+      <c r="F36" s="23"/>
+      <c r="G36" s="23"/>
+      <c r="H36" s="23"/>
+      <c r="I36" s="23"/>
+      <c r="J36" s="23"/>
+      <c r="K36" s="23"/>
+      <c r="L36" s="23"/>
+    </row>
+    <row r="37" spans="1:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
+      <c r="B37" t="s">
         <v>67</v>
       </c>
-      <c r="D37" s="8" t="s">
+      <c r="D37" t="s">
         <v>64</v>
       </c>
-      <c r="E37" s="8" t="s">
+      <c r="E37" t="s">
         <v>58</v>
       </c>
-      <c r="F37" s="8">
+      <c r="F37">
         <v>1250</v>
       </c>
     </row>
-    <row r="38" spans="1:12" outlineLevel="2" x14ac:dyDescent="0.25">
-      <c r="D38" s="8" t="s">
+    <row r="38" spans="1:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25">
+      <c r="D38" t="s">
         <v>64</v>
       </c>
-      <c r="E38" s="8" t="s">
+      <c r="E38" t="s">
         <v>58</v>
       </c>
-      <c r="F38" s="8">
+      <c r="F38">
         <v>500</v>
       </c>
     </row>
-    <row r="39" spans="1:12" outlineLevel="2" x14ac:dyDescent="0.25"/>
-    <row r="40" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25"/>
-    <row r="42" spans="1:12" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:12" hidden="1" outlineLevel="2" x14ac:dyDescent="0.25"/>
+    <row r="40" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="42" spans="1:12" collapsed="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="B42" s="6" t="s">
+      <c r="B42" s="23" t="s">
         <v>95</v>
       </c>
-      <c r="C42" s="6"/>
-      <c r="D42" s="6"/>
-      <c r="E42" s="6"/>
-      <c r="F42" s="6"/>
-      <c r="G42" s="6"/>
-      <c r="H42" s="6"/>
-      <c r="I42" s="6"/>
-      <c r="J42" s="6"/>
-      <c r="K42" s="6"/>
-      <c r="L42" s="6"/>
-    </row>
-    <row r="43" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25"/>
-    <row r="44" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="B44" s="8" t="s">
+      <c r="C42" s="23"/>
+      <c r="D42" s="23"/>
+      <c r="E42" s="23"/>
+      <c r="F42" s="23"/>
+      <c r="G42" s="23"/>
+      <c r="H42" s="23"/>
+      <c r="I42" s="23"/>
+      <c r="J42" s="23"/>
+      <c r="K42" s="23"/>
+      <c r="L42" s="23"/>
+    </row>
+    <row r="43" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="44" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B44" t="s">
         <v>102</v>
       </c>
-      <c r="C44" s="8" t="s">
+      <c r="C44" t="s">
         <v>78</v>
       </c>
-      <c r="D44" s="8" t="s">
+      <c r="D44" t="s">
         <v>5</v>
       </c>
-      <c r="E44" s="8" t="s">
+      <c r="E44" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="45" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="B45" s="8" t="s">
+    <row r="45" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B45" t="s">
         <v>103</v>
       </c>
-      <c r="C45" s="8" t="s">
+      <c r="C45" t="s">
         <v>78</v>
       </c>
-      <c r="D45" s="8" t="s">
+      <c r="D45" t="s">
         <v>5</v>
       </c>
-      <c r="E45" s="8" t="s">
+      <c r="E45" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="46" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="C46" s="8" t="s">
+    <row r="46" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="C46" t="s">
         <v>79</v>
       </c>
-      <c r="D46" s="8" t="s">
+      <c r="D46" t="s">
         <v>5</v>
       </c>
-      <c r="E46" s="8" t="s">
+      <c r="E46" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="47" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25"/>
-    <row r="48" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="B48" s="8" t="s">
+    <row r="47" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="48" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B48" t="s">
         <v>105</v>
       </c>
-      <c r="D48" s="8" t="s">
+      <c r="D48" t="s">
         <v>5</v>
       </c>
-      <c r="E48" s="8" t="s">
+      <c r="E48" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="49" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="D49" s="8" t="s">
+    <row r="49" spans="2:5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="D49" t="s">
         <v>5</v>
       </c>
-      <c r="E49" s="8" t="s">
+      <c r="E49" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="50" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25"/>
-    <row r="51" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25"/>
-    <row r="52" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="B52" s="8" t="s">
+    <row r="50" spans="2:5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="51" spans="2:5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="52" spans="2:5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B52" t="s">
         <v>107</v>
       </c>
-      <c r="D52" s="8" t="s">
+      <c r="D52" t="s">
         <v>13</v>
       </c>
-      <c r="E52" s="8" t="s">
+      <c r="E52" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="53" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="D53" s="8" t="s">
+    <row r="53" spans="2:5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="D53" t="s">
         <v>13</v>
       </c>
-      <c r="E53" s="8" t="s">
+      <c r="E53" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="54" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25"/>
-    <row r="55" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25"/>
-    <row r="56" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="B56" s="8" t="s">
+    <row r="54" spans="2:5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="55" spans="2:5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="56" spans="2:5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B56" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="57" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25"/>
-    <row r="58" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25"/>
-    <row r="59" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="B59" s="8" t="s">
+    <row r="57" spans="2:5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="58" spans="2:5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="59" spans="2:5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B59" t="s">
         <v>110</v>
       </c>
-      <c r="D59" s="8" t="s">
+      <c r="D59" t="s">
         <v>13</v>
       </c>
-      <c r="E59" s="8" t="s">
+      <c r="E59" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="60" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="D60" s="8" t="s">
+    <row r="60" spans="2:5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="D60" t="s">
         <v>13</v>
       </c>
-      <c r="E60" s="8" t="s">
+      <c r="E60" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="61" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25"/>
-    <row r="62" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="B62" s="8" t="s">
+    <row r="61" spans="2:5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="62" spans="2:5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B62" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="63" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25"/>
-    <row r="64" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="B64" s="8" t="s">
+    <row r="63" spans="2:5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="64" spans="2:5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B64" t="s">
         <v>114</v>
       </c>
-      <c r="C64" s="8" t="s">
+      <c r="C64" t="s">
         <v>56</v>
       </c>
-      <c r="D64" s="8" t="s">
+      <c r="D64" t="s">
         <v>5</v>
       </c>
-      <c r="E64" s="11" t="s">
+      <c r="E64" s="5" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="65" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="C65" s="8">
-        <v>1</v>
-      </c>
-      <c r="D65" s="8" t="s">
+    <row r="65" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="C65">
+        <v>1</v>
+      </c>
+      <c r="D65" t="s">
         <v>13</v>
       </c>
-      <c r="E65" s="8" t="s">
+      <c r="E65" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="66" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="C66" s="8">
+    <row r="66" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="C66">
         <v>2</v>
       </c>
-      <c r="D66" s="8" t="s">
+      <c r="D66" t="s">
         <v>13</v>
       </c>
-      <c r="E66" s="8" t="s">
+      <c r="E66" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="67" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25"/>
-    <row r="68" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="B68" s="8" t="s">
+    <row r="67" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="68" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B68" t="s">
         <v>122</v>
       </c>
-      <c r="C68" s="8" t="s">
+      <c r="C68" t="s">
         <v>58</v>
       </c>
-      <c r="D68" s="8" t="s">
+      <c r="D68" t="s">
         <v>6</v>
       </c>
-      <c r="E68" s="8">
+      <c r="E68">
         <v>1000</v>
       </c>
     </row>
-    <row r="69" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="69" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="70" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="71" spans="1:12" ht="15.75" collapsed="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A71" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B71" s="20" t="s">
+        <v>160</v>
+      </c>
+      <c r="C71" s="21"/>
+      <c r="D71" s="21"/>
+      <c r="E71" s="21"/>
+      <c r="F71" s="21"/>
+      <c r="G71" s="21"/>
+      <c r="H71" s="21"/>
+      <c r="I71" s="21"/>
+      <c r="J71" s="21"/>
+      <c r="K71" s="21"/>
+      <c r="L71" s="22"/>
+    </row>
+    <row r="72" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="73" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B73" s="10" t="s">
+        <v>164</v>
+      </c>
+      <c r="C73" s="10"/>
+      <c r="D73" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="E73" s="10" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="74" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B74" s="10"/>
+      <c r="C74" s="10"/>
+      <c r="D74" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="E74" s="10" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="75" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B75" s="10"/>
+      <c r="C75" s="10"/>
+      <c r="D75" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="E75" s="10" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="76" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B76" s="10"/>
+      <c r="C76" s="10"/>
+      <c r="D76" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="E76" s="10" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="77" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B77" s="10"/>
+      <c r="C77" s="10"/>
+      <c r="D77" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="E77" s="10" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="78" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B78" s="10"/>
+      <c r="C78" s="10"/>
+      <c r="D78" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="E78" s="10" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="79" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B79" s="10"/>
+      <c r="C79" s="10"/>
+      <c r="D79" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="E79" s="10" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="80" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B80" s="10"/>
+      <c r="C80" s="10"/>
+      <c r="D80" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="E80" s="10" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="81" spans="2:5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B81" s="10"/>
+      <c r="C81" s="10"/>
+      <c r="D81" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="E81" s="10" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="82" spans="2:5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B82" s="10"/>
+      <c r="C82" s="10"/>
+      <c r="D82" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="E82" s="10" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="83" spans="2:5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B83" s="10"/>
+      <c r="C83" s="10"/>
+      <c r="D83" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="E83" s="10" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="84" spans="2:5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="8">
+    <mergeCell ref="B71:L71"/>
+    <mergeCell ref="B36:L36"/>
+    <mergeCell ref="B42:L42"/>
     <mergeCell ref="B5:L5"/>
     <mergeCell ref="B7:L7"/>
     <mergeCell ref="B12:L12"/>
     <mergeCell ref="B26:L26"/>
     <mergeCell ref="B27:L27"/>
-    <mergeCell ref="B36:L36"/>
-    <mergeCell ref="B42:L42"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2906,374 +3419,2298 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:L43"/>
+  <dimension ref="A1:W102"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.140625" style="8"/>
-    <col min="2" max="2" width="33.140625" style="8" customWidth="1"/>
-    <col min="3" max="3" width="13" style="8" customWidth="1"/>
-    <col min="4" max="4" width="11.140625" style="8" customWidth="1"/>
-    <col min="5" max="5" width="35.7109375" style="8" customWidth="1"/>
-    <col min="6" max="6" width="14.42578125" style="8" customWidth="1"/>
-    <col min="7" max="16384" width="9.140625" style="8"/>
+    <col min="2" max="2" width="33.140625" customWidth="1"/>
+    <col min="3" max="3" width="13" customWidth="1"/>
+    <col min="4" max="4" width="23.140625" customWidth="1"/>
+    <col min="5" max="5" width="35.7109375" customWidth="1"/>
+    <col min="6" max="6" width="14.42578125" customWidth="1"/>
+    <col min="7" max="7" width="11.85546875" customWidth="1"/>
+    <col min="8" max="8" width="17.5703125" customWidth="1"/>
+    <col min="9" max="10" width="13.140625" customWidth="1"/>
+    <col min="13" max="13" width="14" customWidth="1"/>
+    <col min="14" max="14" width="6.7109375" customWidth="1"/>
+    <col min="15" max="15" width="32.140625" customWidth="1"/>
+    <col min="16" max="16" width="9.140625" customWidth="1"/>
+    <col min="17" max="17" width="21.5703125" customWidth="1"/>
+    <col min="18" max="18" width="16" customWidth="1"/>
+    <col min="20" max="20" width="11.140625" customWidth="1"/>
+    <col min="21" max="21" width="15.140625" customWidth="1"/>
+    <col min="22" max="22" width="21.5703125" customWidth="1"/>
+    <col min="23" max="23" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="8" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="8" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="8" t="s">
+      <c r="F1" t="s">
         <v>66</v>
       </c>
-      <c r="G1" s="8" t="s">
+      <c r="G1" t="s">
         <v>81</v>
       </c>
-      <c r="H1" s="8" t="s">
+      <c r="H1" t="s">
         <v>82</v>
       </c>
-      <c r="I1" s="8" t="s">
+      <c r="I1" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="5" spans="1:12" s="9" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="B5" s="7" t="str">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="B5" s="26" t="str">
         <f>'Lvl1'!B5:XFD5</f>
         <v>This row start parsing</v>
       </c>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
-      <c r="H5" s="7"/>
-      <c r="I5" s="7"/>
-      <c r="J5" s="7"/>
-      <c r="K5" s="7"/>
-      <c r="L5" s="7"/>
-    </row>
-    <row r="7" spans="1:12" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C5" s="26"/>
+      <c r="D5" s="26"/>
+      <c r="E5" s="26"/>
+      <c r="F5" s="26"/>
+      <c r="G5" s="26"/>
+      <c r="H5" s="26"/>
+      <c r="I5" s="26"/>
+      <c r="J5" s="26"/>
+      <c r="K5" s="26"/>
+      <c r="L5" s="26"/>
+    </row>
+    <row r="7" spans="1:12" collapsed="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="B7" s="6" t="str">
+      <c r="B7" s="23" t="str">
         <f>'Lvl1'!B12:XFD12</f>
         <v>Example2. Types variation</v>
       </c>
-      <c r="C7" s="6"/>
-      <c r="D7" s="6"/>
-      <c r="E7" s="6"/>
-      <c r="F7" s="6"/>
-      <c r="G7" s="6"/>
-      <c r="H7" s="6"/>
-      <c r="I7" s="6"/>
-      <c r="J7" s="6"/>
-      <c r="K7" s="6"/>
-      <c r="L7" s="6"/>
-    </row>
-    <row r="8" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="8" t="s">
+      <c r="C7" s="23"/>
+      <c r="D7" s="23"/>
+      <c r="E7" s="23"/>
+      <c r="F7" s="23"/>
+      <c r="G7" s="23"/>
+      <c r="H7" s="23"/>
+      <c r="I7" s="23"/>
+      <c r="J7" s="23"/>
+      <c r="K7" s="23"/>
+      <c r="L7" s="23"/>
+    </row>
+    <row r="8" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
         <v>44</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" t="s">
         <v>34</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" t="s">
         <v>5</v>
       </c>
-      <c r="E8" s="8" t="s">
+      <c r="E8" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="C9" s="8" t="s">
+    <row r="9" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="C9" t="s">
         <v>35</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="D9" t="s">
         <v>6</v>
       </c>
-      <c r="E9" s="8">
+      <c r="E9">
         <v>12345</v>
       </c>
     </row>
-    <row r="10" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25"/>
-    <row r="11" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="8" t="s">
+    <row r="10" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="11" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
         <v>45</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="C11" t="s">
         <v>34</v>
       </c>
-      <c r="D11" s="8" t="s">
+      <c r="D11" t="s">
         <v>26</v>
       </c>
-      <c r="E11" s="8" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="C12" s="8" t="s">
+      <c r="E11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="C12" t="s">
         <v>35</v>
       </c>
-      <c r="D12" s="8" t="s">
+      <c r="D12" t="s">
         <v>26</v>
       </c>
-      <c r="E12" s="8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25"/>
-    <row r="14" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="8" t="s">
+      <c r="E12" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="14" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
         <v>46</v>
       </c>
-      <c r="C14" s="8" t="s">
+      <c r="C14" t="s">
         <v>34</v>
       </c>
-      <c r="D14" s="8" t="s">
+      <c r="D14" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="15" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="C15" s="8" t="s">
+    <row r="15" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="C15" t="s">
         <v>35</v>
       </c>
-      <c r="D15" s="8" t="s">
+      <c r="D15" t="s">
         <v>5</v>
       </c>
-      <c r="E15" s="8" t="s">
+      <c r="E15" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="16" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25"/>
-    <row r="18" spans="1:12" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="18" spans="1:15" collapsed="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="B18" s="6" t="str">
+      <c r="B18" s="23" t="str">
         <f>'Lvl1'!B26</f>
         <v>Example3 Alias function</v>
       </c>
-      <c r="C18" s="6"/>
-      <c r="D18" s="6"/>
-      <c r="E18" s="6"/>
-      <c r="F18" s="6"/>
-      <c r="G18" s="6"/>
-      <c r="H18" s="6"/>
-      <c r="I18" s="6"/>
-      <c r="J18" s="6"/>
-      <c r="K18" s="6"/>
-      <c r="L18" s="6"/>
-    </row>
-    <row r="19" spans="1:12" s="9" customFormat="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="C18" s="23"/>
+      <c r="D18" s="23"/>
+      <c r="E18" s="23"/>
+      <c r="F18" s="23"/>
+      <c r="G18" s="23"/>
+      <c r="H18" s="23"/>
+      <c r="I18" s="23"/>
+      <c r="J18" s="23"/>
+      <c r="K18" s="23"/>
+      <c r="L18" s="23"/>
+    </row>
+    <row r="19" spans="1:15" hidden="1" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="B19" s="6" t="str">
+      <c r="B19" s="23" t="str">
         <f>'Lvl1'!B27</f>
         <v>Example3.1 Alias function. Semantics without alias func</v>
       </c>
-      <c r="C19" s="6"/>
-      <c r="D19" s="6"/>
-      <c r="E19" s="6"/>
-      <c r="F19" s="6"/>
-      <c r="G19" s="6"/>
-      <c r="H19" s="6"/>
-      <c r="I19" s="6"/>
-      <c r="J19" s="6"/>
-      <c r="K19" s="6"/>
-      <c r="L19" s="6"/>
-    </row>
-    <row r="20" spans="1:12" ht="15" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.25"/>
-    <row r="21" spans="1:12" ht="15" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.25">
-      <c r="B21" s="8" t="s">
+      <c r="C19" s="23"/>
+      <c r="D19" s="23"/>
+      <c r="E19" s="23"/>
+      <c r="F19" s="23"/>
+      <c r="G19" s="23"/>
+      <c r="H19" s="23"/>
+      <c r="I19" s="23"/>
+      <c r="J19" s="23"/>
+      <c r="K19" s="23"/>
+      <c r="L19" s="23"/>
+    </row>
+    <row r="20" spans="1:15" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.25"/>
+    <row r="21" spans="1:15" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.25">
+      <c r="B21" t="s">
         <v>59</v>
       </c>
-      <c r="C21" s="8" t="s">
+      <c r="C21" t="s">
         <v>56</v>
       </c>
-      <c r="D21" s="8" t="s">
+      <c r="D21" t="s">
         <v>5</v>
       </c>
-      <c r="E21" s="8" t="s">
+      <c r="E21" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="22" spans="1:12" ht="15" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.25">
-      <c r="C22" s="8" t="s">
+    <row r="22" spans="1:15" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.25">
+      <c r="C22" t="s">
         <v>58</v>
       </c>
-      <c r="D22" s="8" t="s">
+      <c r="D22" t="s">
         <v>6</v>
       </c>
-      <c r="E22" s="8">
+      <c r="E22">
         <v>1250</v>
       </c>
     </row>
-    <row r="23" spans="1:12" ht="15" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.25">
-      <c r="B23" s="8" t="s">
+    <row r="23" spans="1:15" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.25">
+      <c r="B23" t="s">
         <v>61</v>
       </c>
-      <c r="C23" s="8" t="s">
+      <c r="C23" t="s">
         <v>56</v>
       </c>
-      <c r="D23" s="8" t="s">
+      <c r="D23" t="s">
         <v>5</v>
       </c>
-      <c r="E23" s="8" t="s">
+      <c r="E23" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="24" spans="1:12" ht="15" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.25">
-      <c r="C24" s="8" t="s">
+    <row r="24" spans="1:15" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.25">
+      <c r="C24" t="s">
         <v>58</v>
       </c>
-      <c r="D24" s="8" t="s">
+      <c r="D24" t="s">
         <v>6</v>
       </c>
-      <c r="E24" s="8">
+      <c r="E24">
         <v>500</v>
       </c>
     </row>
-    <row r="25" spans="1:12" ht="15" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.25"/>
-    <row r="26" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25"/>
-    <row r="27" spans="1:12" s="9" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="8"/>
-    </row>
-    <row r="28" spans="1:12" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:15" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.25">
+      <c r="O25" s="29" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="28" spans="1:15" collapsed="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="B28" s="6" t="s">
+      <c r="B28" s="23" t="s">
         <v>95</v>
       </c>
-      <c r="C28" s="6"/>
-      <c r="D28" s="6"/>
-      <c r="E28" s="6"/>
-      <c r="F28" s="6"/>
-      <c r="G28" s="6"/>
-      <c r="H28" s="6"/>
-      <c r="I28" s="6"/>
-      <c r="J28" s="6"/>
-      <c r="K28" s="6"/>
-      <c r="L28" s="6"/>
-    </row>
-    <row r="29" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25"/>
-    <row r="30" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="8" t="s">
+      <c r="C28" s="23"/>
+      <c r="D28" s="23"/>
+      <c r="E28" s="23"/>
+      <c r="F28" s="23"/>
+      <c r="G28" s="23"/>
+      <c r="H28" s="23"/>
+      <c r="I28" s="23"/>
+      <c r="J28" s="23"/>
+      <c r="K28" s="23"/>
+      <c r="L28" s="23"/>
+    </row>
+    <row r="29" spans="1:15" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="30" spans="1:15" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B30" t="s">
         <v>142</v>
       </c>
-      <c r="C30" s="8" t="s">
+      <c r="C30" t="s">
         <v>78</v>
       </c>
-      <c r="D30" s="8" t="s">
+      <c r="D30" t="s">
         <v>5</v>
       </c>
-      <c r="E30" s="8" t="s">
+      <c r="E30" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="31" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="C31" s="8" t="s">
+    <row r="31" spans="1:15" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="C31" t="s">
         <v>149</v>
       </c>
-      <c r="D31" s="8" t="s">
+      <c r="D31" t="s">
         <v>6</v>
       </c>
-      <c r="E31" s="8">
+      <c r="E31">
         <v>123</v>
       </c>
     </row>
-    <row r="32" spans="1:12" outlineLevel="1" x14ac:dyDescent="0.25"/>
-    <row r="33" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25"/>
-    <row r="34" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="8" t="s">
+    <row r="32" spans="1:15" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="33" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="34" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B34" t="s">
         <v>143</v>
       </c>
-      <c r="C34" s="8" t="s">
+      <c r="C34" t="s">
         <v>150</v>
       </c>
-      <c r="D34" s="8" t="s">
+      <c r="D34" t="s">
         <v>151</v>
       </c>
-      <c r="E34" s="8" t="s">
+      <c r="E34" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="35" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="C35" s="8" t="s">
+    <row r="35" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="C35" t="s">
         <v>152</v>
       </c>
-      <c r="D35" s="8" t="s">
+      <c r="D35" t="s">
         <v>6</v>
       </c>
-      <c r="E35" s="8">
+      <c r="E35">
         <v>123</v>
       </c>
     </row>
-    <row r="36" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25"/>
-    <row r="37" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25"/>
-    <row r="38" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="B38" s="8" t="s">
+    <row r="36" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="37" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="38" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B38" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="39" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="B39" s="8" t="s">
+    <row r="39" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B39" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="40" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25"/>
-    <row r="41" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="B41" s="8" t="s">
+    <row r="40" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="41" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B41" t="s">
         <v>147</v>
       </c>
-      <c r="C41" s="8" t="s">
+      <c r="C41" t="s">
         <v>78</v>
       </c>
-      <c r="D41" s="8" t="s">
+      <c r="D41" t="s">
         <v>5</v>
       </c>
-      <c r="E41" s="8" t="s">
+      <c r="E41" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="42" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="B42" s="8" t="s">
+    <row r="42" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B42" t="s">
         <v>148</v>
       </c>
-      <c r="C42" s="8" t="s">
+      <c r="C42" t="s">
         <v>79</v>
       </c>
-      <c r="D42" s="8" t="s">
+      <c r="D42" t="s">
         <v>6</v>
       </c>
-      <c r="E42" s="8">
+      <c r="E42">
         <v>456</v>
       </c>
     </row>
-    <row r="43" spans="2:5" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="43" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="44" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="45" spans="1:12" ht="15.75" collapsed="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B45" s="20" t="s">
+        <v>160</v>
+      </c>
+      <c r="C45" s="21"/>
+      <c r="D45" s="21"/>
+      <c r="E45" s="21"/>
+      <c r="F45" s="21"/>
+      <c r="G45" s="21"/>
+      <c r="H45" s="21"/>
+      <c r="I45" s="21"/>
+      <c r="J45" s="21"/>
+      <c r="K45" s="21"/>
+      <c r="L45" s="22"/>
+    </row>
+    <row r="46" spans="1:12" ht="15.75" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="47" spans="1:12" ht="15.75" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="30" t="b">
+        <v>1</v>
+      </c>
+      <c r="B47" s="20" t="s">
+        <v>176</v>
+      </c>
+      <c r="C47" s="21"/>
+      <c r="D47" s="21"/>
+      <c r="E47" s="21"/>
+      <c r="F47" s="21"/>
+      <c r="G47" s="21"/>
+      <c r="H47" s="21"/>
+      <c r="I47" s="22"/>
+      <c r="J47" s="18" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="49" spans="2:23" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B49" s="8" t="str">
+        <f>_xlfn.CONCAT("stage",J49)</f>
+        <v>stage0</v>
+      </c>
+      <c r="C49" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="D49" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="E49" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="F49" s="5"/>
+      <c r="G49" s="5"/>
+      <c r="H49" s="5"/>
+      <c r="I49" s="5"/>
+      <c r="J49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="2:23" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B50" s="5"/>
+      <c r="C50" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="D50" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="E50" s="8" cm="1">
+        <f t="array" ref="E50">_xlfn.TAKE(_xlfn._xlws.FILTER($S$54:$S$75,$N$54:$N$75=J50, TRUE), 1)</f>
+        <v>50</v>
+      </c>
+      <c r="F50" s="5"/>
+      <c r="G50" s="5"/>
+      <c r="H50" s="5"/>
+      <c r="I50" s="5"/>
+      <c r="J50">
+        <f>J49</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="2:23" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B51" s="5"/>
+      <c r="C51" s="8" t="s">
+        <v>180</v>
+      </c>
+      <c r="D51" s="5" t="str" cm="1">
+        <f t="array" ref="D51">_xlfn._xlws.FILTER($O$54:$O$75, ($M$54:$M$75=$C51)*($N$54:$N$75=$J51))</f>
+        <v>SeasonLootBoxReward</v>
+      </c>
+      <c r="E51" s="5"/>
+      <c r="F51" s="5"/>
+      <c r="G51" s="5" t="b" cm="1">
+        <f t="array" ref="G51">_xlfn._xlws.FILTER($P$54:$P$75, (ISBLANK($P$54:$P$75)=FALSE)*($M$54:$M$75=$C51)*($N$54:$N$75=$J51), "")</f>
+        <v>0</v>
+      </c>
+      <c r="H51" s="5" t="str" cm="1">
+        <f t="array" ref="H51">_xlfn._xlws.FILTER($Q$54:$Q$75, (ISBLANK($Q$54:$Q$75)=FALSE)*($M$54:$M$75=$C51)*($N$54:$N$75=$J51), "")</f>
+        <v>LootBoxSilver</v>
+      </c>
+      <c r="I51" s="5" t="str" cm="1">
+        <f t="array" ref="I51">_xlfn._xlws.FILTER($R$54:$R$75, (ISBLANK($R$54:$R$75)=FALSE)*($M$54:$M$75=$C51)*($N$54:$N$75=$J51), "")</f>
+        <v/>
+      </c>
+      <c r="J51">
+        <f t="shared" ref="J51:J52" si="0">J50</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="2:23" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B52" s="5"/>
+      <c r="C52" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="D52" s="5" t="str" cm="1">
+        <f t="array" ref="D52">_xlfn._xlws.FILTER($O$54:$O$75, ($M$54:$M$75=$C52)*($N$54:$N$75=$J52))</f>
+        <v>SeasonLootBoxReward</v>
+      </c>
+      <c r="E52" s="5"/>
+      <c r="F52" s="5"/>
+      <c r="G52" s="5" t="b" cm="1">
+        <f t="array" ref="G52">_xlfn._xlws.FILTER($P$54:$P$75, (ISBLANK($P$54:$P$75)=FALSE)*($M$54:$M$75=$C52)*($N$54:$N$75=$J52), "")</f>
+        <v>0</v>
+      </c>
+      <c r="H52" s="5" t="str" cm="1">
+        <f t="array" ref="H52">_xlfn._xlws.FILTER($Q$54:$Q$75, (ISBLANK($Q$54:$Q$75)=FALSE)*($M$54:$M$75=$C52)*($N$54:$N$75=$J52), "")</f>
+        <v>LootBoxGold</v>
+      </c>
+      <c r="I52" s="5" t="str" cm="1">
+        <f t="array" ref="I52">_xlfn._xlws.FILTER($R$54:$R$75, (ISBLANK($R$54:$R$75)=FALSE)*($M$54:$M$75=$C52)*($N$54:$N$75=$J52), "")</f>
+        <v/>
+      </c>
+      <c r="J52">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="M52" s="5"/>
+      <c r="N52" s="5"/>
+      <c r="O52" s="25" t="s">
+        <v>183</v>
+      </c>
+      <c r="P52" s="25"/>
+      <c r="Q52" s="25"/>
+      <c r="R52" s="25"/>
+      <c r="S52" s="5"/>
+      <c r="T52" s="5"/>
+      <c r="U52" s="5"/>
+      <c r="V52" s="5"/>
+      <c r="W52" s="5"/>
+    </row>
+    <row r="53" spans="2:23" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="M53" s="12"/>
+      <c r="N53" s="13" t="s">
+        <v>186</v>
+      </c>
+      <c r="O53" s="13" t="s">
+        <v>187</v>
+      </c>
+      <c r="P53" s="13" t="s">
+        <v>81</v>
+      </c>
+      <c r="Q53" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="R53" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="S53" s="13" t="s">
+        <v>188</v>
+      </c>
+      <c r="T53" s="13" t="s">
+        <v>189</v>
+      </c>
+      <c r="U53" s="13" t="s">
+        <v>190</v>
+      </c>
+      <c r="V53" s="13" t="s">
+        <v>191</v>
+      </c>
+      <c r="W53" s="13" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="54" spans="2:23" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B54" s="8" t="str">
+        <f>_xlfn.CONCAT("stage",J54)</f>
+        <v>stage1</v>
+      </c>
+      <c r="C54" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="D54" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="E54" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="F54" s="5"/>
+      <c r="G54" s="5"/>
+      <c r="H54" s="5"/>
+      <c r="I54" s="5"/>
+      <c r="J54">
+        <v>1</v>
+      </c>
+      <c r="M54" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="N54" s="14">
+        <v>0</v>
+      </c>
+      <c r="O54" s="15" t="s">
+        <v>181</v>
+      </c>
+      <c r="P54" s="15" t="b">
+        <f>T54</f>
+        <v>0</v>
+      </c>
+      <c r="Q54" s="15" t="str">
+        <f>V54</f>
+        <v>LootBoxSilver</v>
+      </c>
+      <c r="R54" s="15"/>
+      <c r="S54" s="27">
+        <v>50</v>
+      </c>
+      <c r="T54" s="16" t="b">
+        <v>0</v>
+      </c>
+      <c r="U54" s="15" t="s">
+        <v>193</v>
+      </c>
+      <c r="V54" s="17" t="s">
+        <v>182</v>
+      </c>
+      <c r="W54" s="15"/>
+    </row>
+    <row r="55" spans="2:23" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B55" s="5"/>
+      <c r="C55" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="D55" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="E55" s="8" cm="1">
+        <f t="array" ref="E55">_xlfn.TAKE(_xlfn._xlws.FILTER($S$54:$S$75,$N$54:$N$75=J55, TRUE), 1)</f>
+        <v>150</v>
+      </c>
+      <c r="F55" s="5"/>
+      <c r="G55" s="5"/>
+      <c r="H55" s="5"/>
+      <c r="I55" s="5"/>
+      <c r="J55">
+        <f>J54</f>
+        <v>1</v>
+      </c>
+      <c r="M55" s="12" t="s">
+        <v>184</v>
+      </c>
+      <c r="N55" s="14">
+        <v>0</v>
+      </c>
+      <c r="O55" s="15" t="s">
+        <v>181</v>
+      </c>
+      <c r="P55" s="15" t="b">
+        <f t="shared" ref="P55:P75" si="1">T55</f>
+        <v>0</v>
+      </c>
+      <c r="Q55" s="15" t="str">
+        <f>V55</f>
+        <v>LootBoxGold</v>
+      </c>
+      <c r="R55" s="15"/>
+      <c r="S55" s="28"/>
+      <c r="T55" s="16" t="b">
+        <v>0</v>
+      </c>
+      <c r="U55" s="15" t="s">
+        <v>193</v>
+      </c>
+      <c r="V55" s="17" t="s">
+        <v>185</v>
+      </c>
+      <c r="W55" s="15"/>
+    </row>
+    <row r="56" spans="2:23" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B56" s="5"/>
+      <c r="C56" s="8" t="s">
+        <v>180</v>
+      </c>
+      <c r="D56" s="5" t="str" cm="1">
+        <f t="array" ref="D56">_xlfn._xlws.FILTER($O$54:$O$75, ($M$54:$M$75=$C56)*($N$54:$N$75=$J56))</f>
+        <v>SeasonWheelTicketsReward</v>
+      </c>
+      <c r="E56" s="5"/>
+      <c r="F56" s="5"/>
+      <c r="G56" s="5" t="b" cm="1">
+        <f t="array" ref="G56">_xlfn._xlws.FILTER($P$54:$P$75, (ISBLANK($P$54:$P$75)=FALSE)*($M$54:$M$75=$C56)*($N$54:$N$75=$J56), "")</f>
+        <v>0</v>
+      </c>
+      <c r="H56" s="5" t="str" cm="1">
+        <f t="array" ref="H56">_xlfn._xlws.FILTER($Q$54:$Q$75, (ISBLANK($Q$54:$Q$75)=FALSE)*($M$54:$M$75=$C56)*($N$54:$N$75=$J56), "")</f>
+        <v>Basic</v>
+      </c>
+      <c r="I56" s="5" cm="1">
+        <f t="array" ref="I56">_xlfn._xlws.FILTER($R$54:$R$75, (ISBLANK($R$54:$R$75)=FALSE)*($M$54:$M$75=$C56)*($N$54:$N$75=$J56), "")</f>
+        <v>1</v>
+      </c>
+      <c r="J56">
+        <f t="shared" ref="J56:J57" si="2">J55</f>
+        <v>1</v>
+      </c>
+      <c r="M56" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="N56" s="14">
+        <v>1</v>
+      </c>
+      <c r="O56" s="15" t="s">
+        <v>194</v>
+      </c>
+      <c r="P56" s="15" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Q56" s="15" t="str">
+        <f>V56</f>
+        <v>Basic</v>
+      </c>
+      <c r="R56" s="15">
+        <f>W56</f>
+        <v>1</v>
+      </c>
+      <c r="S56" s="24">
+        <v>150</v>
+      </c>
+      <c r="T56" s="16" t="b">
+        <v>0</v>
+      </c>
+      <c r="U56" s="15" t="s">
+        <v>196</v>
+      </c>
+      <c r="V56" s="17" t="s">
+        <v>195</v>
+      </c>
+      <c r="W56" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" spans="2:23" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B57" s="5"/>
+      <c r="C57" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="D57" s="5" t="str" cm="1">
+        <f t="array" ref="D57">_xlfn._xlws.FILTER($O$54:$O$75, ($M$54:$M$75=$C57)*($N$54:$N$75=$J57))</f>
+        <v>SeasonCoreRandomBoosterReward</v>
+      </c>
+      <c r="E57" s="5"/>
+      <c r="F57" s="5"/>
+      <c r="G57" s="5" t="b" cm="1">
+        <f t="array" ref="G57">_xlfn._xlws.FILTER($P$54:$P$75, (ISBLANK($P$54:$P$75)=FALSE)*($M$54:$M$75=$C57)*($N$54:$N$75=$J57), "")</f>
+        <v>0</v>
+      </c>
+      <c r="H57" s="5" t="str" cm="1">
+        <f t="array" ref="H57">_xlfn._xlws.FILTER($Q$54:$Q$75, (ISBLANK($Q$54:$Q$75)=FALSE)*($M$54:$M$75=$C57)*($N$54:$N$75=$J57), "")</f>
+        <v>SeasonRandomBooster</v>
+      </c>
+      <c r="I57" s="5" cm="1">
+        <f t="array" ref="I57">_xlfn._xlws.FILTER($R$54:$R$75, (ISBLANK($R$54:$R$75)=FALSE)*($M$54:$M$75=$C57)*($N$54:$N$75=$J57), "")</f>
+        <v>2</v>
+      </c>
+      <c r="J57">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="M57" s="12" t="s">
+        <v>184</v>
+      </c>
+      <c r="N57" s="14">
+        <v>1</v>
+      </c>
+      <c r="O57" s="15" t="s">
+        <v>197</v>
+      </c>
+      <c r="P57" s="15" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Q57" s="15" t="str">
+        <f>V57:V75</f>
+        <v>SeasonRandomBooster</v>
+      </c>
+      <c r="R57" s="15">
+        <f>W57</f>
+        <v>2</v>
+      </c>
+      <c r="S57" s="24"/>
+      <c r="T57" s="16" t="b">
+        <v>0</v>
+      </c>
+      <c r="U57" s="15" t="s">
+        <v>199</v>
+      </c>
+      <c r="V57" s="17" t="s">
+        <v>198</v>
+      </c>
+      <c r="W57" s="17">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="58" spans="2:23" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="M58" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="N58" s="14">
+        <v>2</v>
+      </c>
+      <c r="O58" s="15" t="s">
+        <v>197</v>
+      </c>
+      <c r="P58" s="15" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Q58" s="15" t="str">
+        <f>V58:V76</f>
+        <v>SeasonRandomBooster</v>
+      </c>
+      <c r="R58" s="15">
+        <f>W58</f>
+        <v>2</v>
+      </c>
+      <c r="S58" s="24">
+        <v>250</v>
+      </c>
+      <c r="T58" s="16" t="b">
+        <v>0</v>
+      </c>
+      <c r="U58" s="15" t="s">
+        <v>199</v>
+      </c>
+      <c r="V58" s="17" t="s">
+        <v>198</v>
+      </c>
+      <c r="W58" s="17">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="59" spans="2:23" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B59" s="8" t="str">
+        <f>_xlfn.CONCAT("stage",J59)</f>
+        <v>stage2</v>
+      </c>
+      <c r="C59" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="D59" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="E59" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="F59" s="5"/>
+      <c r="G59" s="5"/>
+      <c r="H59" s="5"/>
+      <c r="I59" s="5"/>
+      <c r="J59">
+        <v>2</v>
+      </c>
+      <c r="M59" s="12" t="s">
+        <v>184</v>
+      </c>
+      <c r="N59" s="14">
+        <v>2</v>
+      </c>
+      <c r="O59" s="15" t="s">
+        <v>200</v>
+      </c>
+      <c r="P59" s="15" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Q59" s="15">
+        <f>W59</f>
+        <v>100</v>
+      </c>
+      <c r="R59" s="15"/>
+      <c r="S59" s="24"/>
+      <c r="T59" s="16" t="b">
+        <v>0</v>
+      </c>
+      <c r="U59" s="15" t="s">
+        <v>201</v>
+      </c>
+      <c r="V59" s="15"/>
+      <c r="W59" s="17">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="60" spans="2:23" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B60" s="5"/>
+      <c r="C60" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="D60" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="E60" s="8" cm="1">
+        <f t="array" ref="E60">_xlfn.TAKE(_xlfn._xlws.FILTER($S$54:$S$75,$N$54:$N$75=J60, TRUE), 1)</f>
+        <v>250</v>
+      </c>
+      <c r="F60" s="5"/>
+      <c r="G60" s="5"/>
+      <c r="H60" s="5"/>
+      <c r="I60" s="5"/>
+      <c r="J60">
+        <f>J59</f>
+        <v>2</v>
+      </c>
+      <c r="M60" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="N60" s="14">
+        <v>3</v>
+      </c>
+      <c r="O60" s="15" t="s">
+        <v>200</v>
+      </c>
+      <c r="P60" s="15" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Q60" s="15">
+        <f>W60</f>
+        <v>500</v>
+      </c>
+      <c r="R60" s="15"/>
+      <c r="S60" s="24">
+        <v>300</v>
+      </c>
+      <c r="T60" s="16" t="b">
+        <v>0</v>
+      </c>
+      <c r="U60" s="15" t="s">
+        <v>201</v>
+      </c>
+      <c r="V60" s="15"/>
+      <c r="W60" s="17">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="61" spans="2:23" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B61" s="5"/>
+      <c r="C61" s="8" t="s">
+        <v>180</v>
+      </c>
+      <c r="D61" s="5" t="str" cm="1">
+        <f t="array" ref="D61">_xlfn._xlws.FILTER($O$54:$O$75, ($M$54:$M$75=$C61)*($N$54:$N$75=$J61))</f>
+        <v>SeasonCoreRandomBoosterReward</v>
+      </c>
+      <c r="E61" s="5"/>
+      <c r="F61" s="5"/>
+      <c r="G61" s="5" t="b" cm="1">
+        <f t="array" ref="G61">_xlfn._xlws.FILTER($P$54:$P$75, (ISBLANK($P$54:$P$75)=FALSE)*($M$54:$M$75=$C61)*($N$54:$N$75=$J61), "")</f>
+        <v>0</v>
+      </c>
+      <c r="H61" s="5" t="str" cm="1">
+        <f t="array" ref="H61">_xlfn._xlws.FILTER($Q$54:$Q$75, (ISBLANK($Q$54:$Q$75)=FALSE)*($M$54:$M$75=$C61)*($N$54:$N$75=$J61), "")</f>
+        <v>SeasonRandomBooster</v>
+      </c>
+      <c r="I61" s="5" cm="1">
+        <f t="array" ref="I61">_xlfn._xlws.FILTER($R$54:$R$75, (ISBLANK($R$54:$R$75)=FALSE)*($M$54:$M$75=$C61)*($N$54:$N$75=$J61), "")</f>
+        <v>2</v>
+      </c>
+      <c r="J61">
+        <f t="shared" ref="J61:J62" si="3">J60</f>
+        <v>2</v>
+      </c>
+      <c r="M61" s="12" t="s">
+        <v>184</v>
+      </c>
+      <c r="N61" s="14">
+        <v>3</v>
+      </c>
+      <c r="O61" s="15" t="s">
+        <v>181</v>
+      </c>
+      <c r="P61" s="15" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Q61" s="15" t="str">
+        <f t="shared" ref="Q61:Q64" si="4">V61</f>
+        <v>LootBoxSilver</v>
+      </c>
+      <c r="R61" s="15"/>
+      <c r="S61" s="24"/>
+      <c r="T61" s="16" t="b">
+        <v>0</v>
+      </c>
+      <c r="U61" s="15" t="s">
+        <v>193</v>
+      </c>
+      <c r="V61" s="17" t="s">
+        <v>182</v>
+      </c>
+      <c r="W61" s="15"/>
+    </row>
+    <row r="62" spans="2:23" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B62" s="5"/>
+      <c r="C62" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="D62" s="5" t="str" cm="1">
+        <f t="array" ref="D62">_xlfn._xlws.FILTER($O$54:$O$75, ($M$54:$M$75=$C62)*($N$54:$N$75=$J62))</f>
+        <v>SeasonHardReward</v>
+      </c>
+      <c r="E62" s="5"/>
+      <c r="F62" s="5"/>
+      <c r="G62" s="5" t="b" cm="1">
+        <f t="array" ref="G62">_xlfn._xlws.FILTER($P$54:$P$75, (ISBLANK($P$54:$P$75)=FALSE)*($M$54:$M$75=$C62)*($N$54:$N$75=$J62), "")</f>
+        <v>0</v>
+      </c>
+      <c r="H62" s="5" cm="1">
+        <f t="array" ref="H62">_xlfn._xlws.FILTER($Q$54:$Q$75, (ISBLANK($Q$54:$Q$75)=FALSE)*($M$54:$M$75=$C62)*($N$54:$N$75=$J62), "")</f>
+        <v>100</v>
+      </c>
+      <c r="I62" s="5" t="str" cm="1">
+        <f t="array" ref="I62">_xlfn._xlws.FILTER($R$54:$R$75, (ISBLANK($R$54:$R$75)=FALSE)*($M$54:$M$75=$C62)*($N$54:$N$75=$J62), "")</f>
+        <v/>
+      </c>
+      <c r="J62">
+        <f t="shared" si="3"/>
+        <v>2</v>
+      </c>
+      <c r="M62" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="N62" s="14">
+        <v>4</v>
+      </c>
+      <c r="O62" s="15" t="s">
+        <v>181</v>
+      </c>
+      <c r="P62" s="15" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Q62" s="15" t="str">
+        <f t="shared" si="4"/>
+        <v>LootBoxSilver</v>
+      </c>
+      <c r="R62" s="15"/>
+      <c r="S62" s="24">
+        <v>350</v>
+      </c>
+      <c r="T62" s="16" t="b">
+        <v>0</v>
+      </c>
+      <c r="U62" s="15" t="s">
+        <v>193</v>
+      </c>
+      <c r="V62" s="17" t="s">
+        <v>182</v>
+      </c>
+      <c r="W62" s="15"/>
+    </row>
+    <row r="63" spans="2:23" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="M63" s="12" t="s">
+        <v>184</v>
+      </c>
+      <c r="N63" s="14">
+        <v>4</v>
+      </c>
+      <c r="O63" s="15" t="s">
+        <v>181</v>
+      </c>
+      <c r="P63" s="15" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Q63" s="15" t="str">
+        <f t="shared" si="4"/>
+        <v>LootBoxGold</v>
+      </c>
+      <c r="R63" s="15"/>
+      <c r="S63" s="24"/>
+      <c r="T63" s="16" t="b">
+        <v>0</v>
+      </c>
+      <c r="U63" s="15" t="s">
+        <v>193</v>
+      </c>
+      <c r="V63" s="17" t="s">
+        <v>185</v>
+      </c>
+      <c r="W63" s="15"/>
+    </row>
+    <row r="64" spans="2:23" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B64" s="8" t="str">
+        <f>_xlfn.CONCAT("stage",J64)</f>
+        <v>stage3</v>
+      </c>
+      <c r="C64" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="D64" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="E64" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="F64" s="5"/>
+      <c r="G64" s="5"/>
+      <c r="H64" s="5"/>
+      <c r="I64" s="5"/>
+      <c r="J64">
+        <v>3</v>
+      </c>
+      <c r="M64" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="N64" s="14">
+        <v>5</v>
+      </c>
+      <c r="O64" s="15" t="s">
+        <v>181</v>
+      </c>
+      <c r="P64" s="15" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Q64" s="15" t="str">
+        <f t="shared" si="4"/>
+        <v>LootBoxGold</v>
+      </c>
+      <c r="R64" s="15"/>
+      <c r="S64" s="24">
+        <v>400</v>
+      </c>
+      <c r="T64" s="16" t="b">
+        <v>0</v>
+      </c>
+      <c r="U64" s="15" t="s">
+        <v>193</v>
+      </c>
+      <c r="V64" s="17" t="s">
+        <v>185</v>
+      </c>
+      <c r="W64" s="15"/>
+    </row>
+    <row r="65" spans="2:23" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B65" s="5"/>
+      <c r="C65" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="D65" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="E65" s="8" cm="1">
+        <f t="array" ref="E65">_xlfn.TAKE(_xlfn._xlws.FILTER($S$54:$S$75,$N$54:$N$75=J65, TRUE), 1)</f>
+        <v>300</v>
+      </c>
+      <c r="F65" s="5"/>
+      <c r="G65" s="5"/>
+      <c r="H65" s="5"/>
+      <c r="I65" s="5"/>
+      <c r="J65">
+        <f>J64</f>
+        <v>3</v>
+      </c>
+      <c r="M65" s="12" t="s">
+        <v>184</v>
+      </c>
+      <c r="N65" s="14">
+        <v>5</v>
+      </c>
+      <c r="O65" s="15" t="s">
+        <v>194</v>
+      </c>
+      <c r="P65" s="15" t="b">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="Q65" s="15" t="str">
+        <f>V65</f>
+        <v>Premium</v>
+      </c>
+      <c r="R65" s="15">
+        <f>W65</f>
+        <v>1</v>
+      </c>
+      <c r="S65" s="24"/>
+      <c r="T65" s="16" t="b">
+        <v>1</v>
+      </c>
+      <c r="U65" s="15" t="s">
+        <v>196</v>
+      </c>
+      <c r="V65" s="17" t="s">
+        <v>202</v>
+      </c>
+      <c r="W65" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="66" spans="2:23" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B66" s="5"/>
+      <c r="C66" s="8" t="s">
+        <v>180</v>
+      </c>
+      <c r="D66" s="5" t="str" cm="1">
+        <f t="array" ref="D66">_xlfn._xlws.FILTER($O$54:$O$75, ($M$54:$M$75=$C66)*($N$54:$N$75=$J66))</f>
+        <v>SeasonHardReward</v>
+      </c>
+      <c r="E66" s="5"/>
+      <c r="F66" s="5"/>
+      <c r="G66" s="5" t="b" cm="1">
+        <f t="array" ref="G66">_xlfn._xlws.FILTER($P$54:$P$75, (ISBLANK($P$54:$P$75)=FALSE)*($M$54:$M$75=$C66)*($N$54:$N$75=$J66), "")</f>
+        <v>0</v>
+      </c>
+      <c r="H66" s="5" cm="1">
+        <f t="array" ref="H66">_xlfn._xlws.FILTER($Q$54:$Q$75, (ISBLANK($Q$54:$Q$75)=FALSE)*($M$54:$M$75=$C66)*($N$54:$N$75=$J66), "")</f>
+        <v>500</v>
+      </c>
+      <c r="I66" s="5" t="str" cm="1">
+        <f t="array" ref="I66">_xlfn._xlws.FILTER($R$54:$R$75, (ISBLANK($R$54:$R$75)=FALSE)*($M$54:$M$75=$C66)*($N$54:$N$75=$J66), "")</f>
+        <v/>
+      </c>
+      <c r="J66">
+        <f t="shared" ref="J66:J67" si="5">J65</f>
+        <v>3</v>
+      </c>
+      <c r="M66" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="N66" s="14">
+        <v>6</v>
+      </c>
+      <c r="O66" s="15" t="s">
+        <v>197</v>
+      </c>
+      <c r="P66" s="15" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Q66" s="15" t="str">
+        <f>V66:V84</f>
+        <v>SeasonRandomBooster</v>
+      </c>
+      <c r="R66" s="15">
+        <f>W66</f>
+        <v>4</v>
+      </c>
+      <c r="S66" s="24">
+        <v>450</v>
+      </c>
+      <c r="T66" s="16" t="b">
+        <v>0</v>
+      </c>
+      <c r="U66" s="15" t="s">
+        <v>199</v>
+      </c>
+      <c r="V66" s="17" t="s">
+        <v>198</v>
+      </c>
+      <c r="W66" s="17">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="67" spans="2:23" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B67" s="5"/>
+      <c r="C67" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="D67" s="5" t="str" cm="1">
+        <f t="array" ref="D67">_xlfn._xlws.FILTER($O$54:$O$75, ($M$54:$M$75=$C67)*($N$54:$N$75=$J67))</f>
+        <v>SeasonLootBoxReward</v>
+      </c>
+      <c r="E67" s="5"/>
+      <c r="F67" s="5"/>
+      <c r="G67" s="5" t="b" cm="1">
+        <f t="array" ref="G67">_xlfn._xlws.FILTER($P$54:$P$75, (ISBLANK($P$54:$P$75)=FALSE)*($M$54:$M$75=$C67)*($N$54:$N$75=$J67), "")</f>
+        <v>0</v>
+      </c>
+      <c r="H67" s="5" t="str" cm="1">
+        <f t="array" ref="H67">_xlfn._xlws.FILTER($Q$54:$Q$75, (ISBLANK($Q$54:$Q$75)=FALSE)*($M$54:$M$75=$C67)*($N$54:$N$75=$J67), "")</f>
+        <v>LootBoxSilver</v>
+      </c>
+      <c r="I67" s="5" t="str" cm="1">
+        <f t="array" ref="I67">_xlfn._xlws.FILTER($R$54:$R$75, (ISBLANK($R$54:$R$75)=FALSE)*($M$54:$M$75=$C67)*($N$54:$N$75=$J67), "")</f>
+        <v/>
+      </c>
+      <c r="J67">
+        <f t="shared" si="5"/>
+        <v>3</v>
+      </c>
+      <c r="M67" s="12" t="s">
+        <v>184</v>
+      </c>
+      <c r="N67" s="14">
+        <v>6</v>
+      </c>
+      <c r="O67" s="15" t="s">
+        <v>200</v>
+      </c>
+      <c r="P67" s="15" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Q67" s="15">
+        <f t="shared" ref="Q67:Q68" si="6">W67</f>
+        <v>100</v>
+      </c>
+      <c r="R67" s="15"/>
+      <c r="S67" s="24"/>
+      <c r="T67" s="16" t="b">
+        <v>0</v>
+      </c>
+      <c r="U67" s="15" t="s">
+        <v>201</v>
+      </c>
+      <c r="V67" s="15"/>
+      <c r="W67" s="17">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="68" spans="2:23" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="M68" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="N68" s="14">
+        <v>7</v>
+      </c>
+      <c r="O68" s="15" t="s">
+        <v>200</v>
+      </c>
+      <c r="P68" s="15" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Q68" s="15">
+        <f t="shared" si="6"/>
+        <v>100</v>
+      </c>
+      <c r="R68" s="15"/>
+      <c r="S68" s="24">
+        <v>500</v>
+      </c>
+      <c r="T68" s="16" t="b">
+        <v>0</v>
+      </c>
+      <c r="U68" s="15" t="s">
+        <v>201</v>
+      </c>
+      <c r="V68" s="15"/>
+      <c r="W68" s="17">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="69" spans="2:23" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B69" s="8" t="str">
+        <f>_xlfn.CONCAT("stage",J69)</f>
+        <v>stage4</v>
+      </c>
+      <c r="C69" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="D69" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="E69" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="F69" s="5"/>
+      <c r="G69" s="5"/>
+      <c r="H69" s="5"/>
+      <c r="I69" s="5"/>
+      <c r="J69">
+        <v>4</v>
+      </c>
+      <c r="M69" s="12" t="s">
+        <v>184</v>
+      </c>
+      <c r="N69" s="14">
+        <v>7</v>
+      </c>
+      <c r="O69" s="15" t="s">
+        <v>181</v>
+      </c>
+      <c r="P69" s="15" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Q69" s="15" t="str">
+        <f>V69</f>
+        <v>LootBoxGold</v>
+      </c>
+      <c r="R69" s="15"/>
+      <c r="S69" s="24"/>
+      <c r="T69" s="16" t="b">
+        <v>0</v>
+      </c>
+      <c r="U69" s="15" t="s">
+        <v>193</v>
+      </c>
+      <c r="V69" s="17" t="s">
+        <v>185</v>
+      </c>
+      <c r="W69" s="15"/>
+    </row>
+    <row r="70" spans="2:23" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B70" s="5"/>
+      <c r="C70" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="D70" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="E70" s="8" cm="1">
+        <f t="array" ref="E70">_xlfn.TAKE(_xlfn._xlws.FILTER($S$54:$S$75,$N$54:$N$75=J70, TRUE), 1)</f>
+        <v>350</v>
+      </c>
+      <c r="F70" s="5"/>
+      <c r="G70" s="5"/>
+      <c r="H70" s="5"/>
+      <c r="I70" s="5"/>
+      <c r="J70">
+        <f>J69</f>
+        <v>4</v>
+      </c>
+      <c r="M70" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="N70" s="14">
+        <v>8</v>
+      </c>
+      <c r="O70" s="15" t="s">
+        <v>194</v>
+      </c>
+      <c r="P70" s="15" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Q70" s="15" t="str">
+        <f>V70</f>
+        <v>Basic</v>
+      </c>
+      <c r="R70" s="15">
+        <f>W70</f>
+        <v>1</v>
+      </c>
+      <c r="S70" s="24">
+        <v>550</v>
+      </c>
+      <c r="T70" s="16" t="b">
+        <v>0</v>
+      </c>
+      <c r="U70" s="15" t="s">
+        <v>196</v>
+      </c>
+      <c r="V70" s="17" t="s">
+        <v>195</v>
+      </c>
+      <c r="W70" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71" spans="2:23" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B71" s="5"/>
+      <c r="C71" s="8" t="s">
+        <v>180</v>
+      </c>
+      <c r="D71" s="5" t="str" cm="1">
+        <f t="array" ref="D71">_xlfn._xlws.FILTER($O$54:$O$75, ($M$54:$M$75=$C71)*($N$54:$N$75=$J71))</f>
+        <v>SeasonLootBoxReward</v>
+      </c>
+      <c r="E71" s="5"/>
+      <c r="F71" s="5"/>
+      <c r="G71" s="5" t="b" cm="1">
+        <f t="array" ref="G71">_xlfn._xlws.FILTER($P$54:$P$75, (ISBLANK($P$54:$P$75)=FALSE)*($M$54:$M$75=$C71)*($N$54:$N$75=$J71), "")</f>
+        <v>0</v>
+      </c>
+      <c r="H71" s="5" t="str" cm="1">
+        <f t="array" ref="H71">_xlfn._xlws.FILTER($Q$54:$Q$75, (ISBLANK($Q$54:$Q$75)=FALSE)*($M$54:$M$75=$C71)*($N$54:$N$75=$J71), "")</f>
+        <v>LootBoxSilver</v>
+      </c>
+      <c r="I71" s="5" t="str" cm="1">
+        <f t="array" ref="I71">_xlfn._xlws.FILTER($R$54:$R$75, (ISBLANK($R$54:$R$75)=FALSE)*($M$54:$M$75=$C71)*($N$54:$N$75=$J71), "")</f>
+        <v/>
+      </c>
+      <c r="J71">
+        <f t="shared" ref="J71:J72" si="7">J70</f>
+        <v>4</v>
+      </c>
+      <c r="M71" s="12" t="s">
+        <v>184</v>
+      </c>
+      <c r="N71" s="14">
+        <v>8</v>
+      </c>
+      <c r="O71" s="15" t="s">
+        <v>197</v>
+      </c>
+      <c r="P71" s="15" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Q71" s="15" t="str">
+        <f>V71:V89</f>
+        <v>SeasonRandomBooster</v>
+      </c>
+      <c r="R71" s="15">
+        <f>W71</f>
+        <v>5</v>
+      </c>
+      <c r="S71" s="24"/>
+      <c r="T71" s="16" t="b">
+        <v>0</v>
+      </c>
+      <c r="U71" s="15" t="s">
+        <v>199</v>
+      </c>
+      <c r="V71" s="17" t="s">
+        <v>198</v>
+      </c>
+      <c r="W71" s="17">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="72" spans="2:23" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B72" s="5"/>
+      <c r="C72" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="D72" s="5" t="str" cm="1">
+        <f t="array" ref="D72">_xlfn._xlws.FILTER($O$54:$O$75, ($M$54:$M$75=$C72)*($N$54:$N$75=$J72))</f>
+        <v>SeasonLootBoxReward</v>
+      </c>
+      <c r="E72" s="5"/>
+      <c r="F72" s="5"/>
+      <c r="G72" s="5" t="b" cm="1">
+        <f t="array" ref="G72">_xlfn._xlws.FILTER($P$54:$P$75, (ISBLANK($P$54:$P$75)=FALSE)*($M$54:$M$75=$C72)*($N$54:$N$75=$J72), "")</f>
+        <v>0</v>
+      </c>
+      <c r="H72" s="5" t="str" cm="1">
+        <f t="array" ref="H72">_xlfn._xlws.FILTER($Q$54:$Q$75, (ISBLANK($Q$54:$Q$75)=FALSE)*($M$54:$M$75=$C72)*($N$54:$N$75=$J72), "")</f>
+        <v>LootBoxGold</v>
+      </c>
+      <c r="I72" s="5" t="str" cm="1">
+        <f t="array" ref="I72">_xlfn._xlws.FILTER($R$54:$R$75, (ISBLANK($R$54:$R$75)=FALSE)*($M$54:$M$75=$C72)*($N$54:$N$75=$J72), "")</f>
+        <v/>
+      </c>
+      <c r="J72">
+        <f t="shared" si="7"/>
+        <v>4</v>
+      </c>
+      <c r="M72" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="N72" s="14">
+        <v>9</v>
+      </c>
+      <c r="O72" s="15" t="s">
+        <v>194</v>
+      </c>
+      <c r="P72" s="15" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Q72" s="15" t="str">
+        <f>V72</f>
+        <v>Basic</v>
+      </c>
+      <c r="R72" s="15">
+        <f>W72</f>
+        <v>1</v>
+      </c>
+      <c r="S72" s="24">
+        <v>600</v>
+      </c>
+      <c r="T72" s="16" t="b">
+        <v>0</v>
+      </c>
+      <c r="U72" s="15" t="s">
+        <v>196</v>
+      </c>
+      <c r="V72" s="17" t="s">
+        <v>195</v>
+      </c>
+      <c r="W72" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73" spans="2:23" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="M73" s="12" t="s">
+        <v>184</v>
+      </c>
+      <c r="N73" s="14">
+        <v>9</v>
+      </c>
+      <c r="O73" s="15" t="s">
+        <v>181</v>
+      </c>
+      <c r="P73" s="15" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Q73" s="15" t="str">
+        <f>V73</f>
+        <v>LootBoxGold</v>
+      </c>
+      <c r="R73" s="15"/>
+      <c r="S73" s="24"/>
+      <c r="T73" s="16" t="b">
+        <v>0</v>
+      </c>
+      <c r="U73" s="15" t="s">
+        <v>193</v>
+      </c>
+      <c r="V73" s="17" t="s">
+        <v>185</v>
+      </c>
+      <c r="W73" s="15"/>
+    </row>
+    <row r="74" spans="2:23" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B74" s="8" t="str">
+        <f>_xlfn.CONCAT("stage",J74)</f>
+        <v>stage5</v>
+      </c>
+      <c r="C74" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="D74" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="E74" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="F74" s="5"/>
+      <c r="G74" s="5"/>
+      <c r="H74" s="5"/>
+      <c r="I74" s="5"/>
+      <c r="J74">
+        <v>5</v>
+      </c>
+      <c r="M74" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="N74" s="14">
+        <v>10</v>
+      </c>
+      <c r="O74" s="15" t="s">
+        <v>197</v>
+      </c>
+      <c r="P74" s="15" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Q74" s="15" t="str">
+        <f t="shared" ref="Q74:Q75" si="8">V74:V92</f>
+        <v>SeasonRandomBooster</v>
+      </c>
+      <c r="R74" s="15">
+        <f t="shared" ref="R74:R75" si="9">W74</f>
+        <v>3</v>
+      </c>
+      <c r="S74" s="24">
+        <v>650</v>
+      </c>
+      <c r="T74" s="16" t="b">
+        <v>0</v>
+      </c>
+      <c r="U74" s="15" t="s">
+        <v>199</v>
+      </c>
+      <c r="V74" s="17" t="s">
+        <v>198</v>
+      </c>
+      <c r="W74" s="17">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="75" spans="2:23" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B75" s="5"/>
+      <c r="C75" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="D75" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="E75" s="8" cm="1">
+        <f t="array" ref="E75">_xlfn.TAKE(_xlfn._xlws.FILTER($S$54:$S$75,$N$54:$N$75=J75, TRUE), 1)</f>
+        <v>400</v>
+      </c>
+      <c r="F75" s="5"/>
+      <c r="G75" s="5"/>
+      <c r="H75" s="5"/>
+      <c r="I75" s="5"/>
+      <c r="J75">
+        <f>J74</f>
+        <v>5</v>
+      </c>
+      <c r="M75" s="12" t="s">
+        <v>184</v>
+      </c>
+      <c r="N75" s="14">
+        <v>10</v>
+      </c>
+      <c r="O75" s="15" t="s">
+        <v>197</v>
+      </c>
+      <c r="P75" s="15" t="b">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="Q75" s="15" t="str">
+        <f t="shared" si="8"/>
+        <v>SeasonRandomBooster</v>
+      </c>
+      <c r="R75" s="15">
+        <f t="shared" si="9"/>
+        <v>5</v>
+      </c>
+      <c r="S75" s="24"/>
+      <c r="T75" s="16" t="b">
+        <v>1</v>
+      </c>
+      <c r="U75" s="15" t="s">
+        <v>199</v>
+      </c>
+      <c r="V75" s="17" t="s">
+        <v>198</v>
+      </c>
+      <c r="W75" s="17">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="76" spans="2:23" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B76" s="5"/>
+      <c r="C76" s="8" t="s">
+        <v>180</v>
+      </c>
+      <c r="D76" s="5" t="str" cm="1">
+        <f t="array" ref="D76">_xlfn._xlws.FILTER($O$54:$O$75, ($M$54:$M$75=$C76)*($N$54:$N$75=$J76))</f>
+        <v>SeasonLootBoxReward</v>
+      </c>
+      <c r="E76" s="5"/>
+      <c r="F76" s="5"/>
+      <c r="G76" s="5" t="b" cm="1">
+        <f t="array" ref="G76">_xlfn._xlws.FILTER($P$54:$P$75, (ISBLANK($P$54:$P$75)=FALSE)*($M$54:$M$75=$C76)*($N$54:$N$75=$J76), "")</f>
+        <v>0</v>
+      </c>
+      <c r="H76" s="5" t="str" cm="1">
+        <f t="array" ref="H76">_xlfn._xlws.FILTER($Q$54:$Q$75, (ISBLANK($Q$54:$Q$75)=FALSE)*($M$54:$M$75=$C76)*($N$54:$N$75=$J76), "")</f>
+        <v>LootBoxGold</v>
+      </c>
+      <c r="I76" s="5" t="str" cm="1">
+        <f t="array" ref="I76">_xlfn._xlws.FILTER($R$54:$R$75, (ISBLANK($R$54:$R$75)=FALSE)*($M$54:$M$75=$C76)*($N$54:$N$75=$J76), "")</f>
+        <v/>
+      </c>
+      <c r="J76">
+        <f t="shared" ref="J76:J77" si="10">J75</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="77" spans="2:23" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B77" s="5"/>
+      <c r="C77" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="D77" s="5" t="str" cm="1">
+        <f t="array" ref="D77">_xlfn._xlws.FILTER($O$54:$O$75, ($M$54:$M$75=$C77)*($N$54:$N$75=$J77))</f>
+        <v>SeasonWheelTicketsReward</v>
+      </c>
+      <c r="E77" s="5"/>
+      <c r="F77" s="5"/>
+      <c r="G77" s="5" t="b" cm="1">
+        <f t="array" ref="G77">_xlfn._xlws.FILTER($P$54:$P$75, (ISBLANK($P$54:$P$75)=FALSE)*($M$54:$M$75=$C77)*($N$54:$N$75=$J77), "")</f>
+        <v>1</v>
+      </c>
+      <c r="H77" s="5" t="str" cm="1">
+        <f t="array" ref="H77">_xlfn._xlws.FILTER($Q$54:$Q$75, (ISBLANK($Q$54:$Q$75)=FALSE)*($M$54:$M$75=$C77)*($N$54:$N$75=$J77), "")</f>
+        <v>Premium</v>
+      </c>
+      <c r="I77" s="5" cm="1">
+        <f t="array" ref="I77">_xlfn._xlws.FILTER($R$54:$R$75, (ISBLANK($R$54:$R$75)=FALSE)*($M$54:$M$75=$C77)*($N$54:$N$75=$J77), "")</f>
+        <v>1</v>
+      </c>
+      <c r="J77">
+        <f t="shared" si="10"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="78" spans="2:23" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="79" spans="2:23" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B79" s="8" t="str">
+        <f>_xlfn.CONCAT("stage",J79)</f>
+        <v>stage6</v>
+      </c>
+      <c r="C79" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="D79" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="E79" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="F79" s="5"/>
+      <c r="G79" s="5"/>
+      <c r="H79" s="5"/>
+      <c r="I79" s="5"/>
+      <c r="J79">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="80" spans="2:23" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B80" s="5"/>
+      <c r="C80" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="D80" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="E80" s="8" cm="1">
+        <f t="array" ref="E80">_xlfn.TAKE(_xlfn._xlws.FILTER($S$54:$S$75,$N$54:$N$75=J80, TRUE), 1)</f>
+        <v>450</v>
+      </c>
+      <c r="F80" s="5"/>
+      <c r="G80" s="5"/>
+      <c r="H80" s="5"/>
+      <c r="I80" s="5"/>
+      <c r="J80">
+        <f>J79</f>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="81" spans="2:10" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B81" s="5"/>
+      <c r="C81" s="8" t="s">
+        <v>180</v>
+      </c>
+      <c r="D81" s="5" t="str" cm="1">
+        <f t="array" ref="D81">_xlfn._xlws.FILTER($O$54:$O$75, ($M$54:$M$75=$C81)*($N$54:$N$75=$J81))</f>
+        <v>SeasonCoreRandomBoosterReward</v>
+      </c>
+      <c r="E81" s="5"/>
+      <c r="F81" s="5"/>
+      <c r="G81" s="5" t="b" cm="1">
+        <f t="array" ref="G81">_xlfn._xlws.FILTER($P$54:$P$75, (ISBLANK($P$54:$P$75)=FALSE)*($M$54:$M$75=$C81)*($N$54:$N$75=$J81), "")</f>
+        <v>0</v>
+      </c>
+      <c r="H81" s="5" t="str" cm="1">
+        <f t="array" ref="H81">_xlfn._xlws.FILTER($Q$54:$Q$75, (ISBLANK($Q$54:$Q$75)=FALSE)*($M$54:$M$75=$C81)*($N$54:$N$75=$J81), "")</f>
+        <v>SeasonRandomBooster</v>
+      </c>
+      <c r="I81" s="5" cm="1">
+        <f t="array" ref="I81">_xlfn._xlws.FILTER($R$54:$R$75, (ISBLANK($R$54:$R$75)=FALSE)*($M$54:$M$75=$C81)*($N$54:$N$75=$J81), "")</f>
+        <v>4</v>
+      </c>
+      <c r="J81">
+        <f t="shared" ref="J81:J82" si="11">J80</f>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="82" spans="2:10" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B82" s="5"/>
+      <c r="C82" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="D82" s="5" t="str" cm="1">
+        <f t="array" ref="D82">_xlfn._xlws.FILTER($O$54:$O$75, ($M$54:$M$75=$C82)*($N$54:$N$75=$J82))</f>
+        <v>SeasonHardReward</v>
+      </c>
+      <c r="E82" s="5"/>
+      <c r="F82" s="5"/>
+      <c r="G82" s="5" t="b" cm="1">
+        <f t="array" ref="G82">_xlfn._xlws.FILTER($P$54:$P$75, (ISBLANK($P$54:$P$75)=FALSE)*($M$54:$M$75=$C82)*($N$54:$N$75=$J82), "")</f>
+        <v>0</v>
+      </c>
+      <c r="H82" s="5" cm="1">
+        <f t="array" ref="H82">_xlfn._xlws.FILTER($Q$54:$Q$75, (ISBLANK($Q$54:$Q$75)=FALSE)*($M$54:$M$75=$C82)*($N$54:$N$75=$J82), "")</f>
+        <v>100</v>
+      </c>
+      <c r="I82" s="5" t="str" cm="1">
+        <f t="array" ref="I82">_xlfn._xlws.FILTER($R$54:$R$75, (ISBLANK($R$54:$R$75)=FALSE)*($M$54:$M$75=$C82)*($N$54:$N$75=$J82), "")</f>
+        <v/>
+      </c>
+      <c r="J82">
+        <f t="shared" si="11"/>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="83" spans="2:10" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="84" spans="2:10" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B84" s="8" t="str">
+        <f>_xlfn.CONCAT("stage",J84)</f>
+        <v>stage7</v>
+      </c>
+      <c r="C84" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="D84" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="E84" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="F84" s="5"/>
+      <c r="G84" s="5"/>
+      <c r="H84" s="5"/>
+      <c r="I84" s="5"/>
+      <c r="J84">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="85" spans="2:10" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B85" s="5"/>
+      <c r="C85" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="D85" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="E85" s="8" cm="1">
+        <f t="array" ref="E85">_xlfn.TAKE(_xlfn._xlws.FILTER($S$54:$S$75,$N$54:$N$75=J85, TRUE), 1)</f>
+        <v>500</v>
+      </c>
+      <c r="F85" s="5"/>
+      <c r="G85" s="5"/>
+      <c r="H85" s="5"/>
+      <c r="I85" s="5"/>
+      <c r="J85">
+        <f>J84</f>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="86" spans="2:10" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B86" s="5"/>
+      <c r="C86" s="8" t="s">
+        <v>180</v>
+      </c>
+      <c r="D86" s="5" t="str" cm="1">
+        <f t="array" ref="D86">_xlfn._xlws.FILTER($O$54:$O$75, ($M$54:$M$75=$C86)*($N$54:$N$75=$J86))</f>
+        <v>SeasonHardReward</v>
+      </c>
+      <c r="E86" s="5"/>
+      <c r="F86" s="5"/>
+      <c r="G86" s="5" t="b" cm="1">
+        <f t="array" ref="G86">_xlfn._xlws.FILTER($P$54:$P$75, (ISBLANK($P$54:$P$75)=FALSE)*($M$54:$M$75=$C86)*($N$54:$N$75=$J86), "")</f>
+        <v>0</v>
+      </c>
+      <c r="H86" s="5" cm="1">
+        <f t="array" ref="H86">_xlfn._xlws.FILTER($Q$54:$Q$75, (ISBLANK($Q$54:$Q$75)=FALSE)*($M$54:$M$75=$C86)*($N$54:$N$75=$J86), "")</f>
+        <v>100</v>
+      </c>
+      <c r="I86" s="5" t="str" cm="1">
+        <f t="array" ref="I86">_xlfn._xlws.FILTER($R$54:$R$75, (ISBLANK($R$54:$R$75)=FALSE)*($M$54:$M$75=$C86)*($N$54:$N$75=$J86), "")</f>
+        <v/>
+      </c>
+      <c r="J86">
+        <f t="shared" ref="J86:J87" si="12">J85</f>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="87" spans="2:10" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B87" s="5"/>
+      <c r="C87" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="D87" s="5" t="str" cm="1">
+        <f t="array" ref="D87">_xlfn._xlws.FILTER($O$54:$O$75, ($M$54:$M$75=$C87)*($N$54:$N$75=$J87))</f>
+        <v>SeasonLootBoxReward</v>
+      </c>
+      <c r="E87" s="5"/>
+      <c r="F87" s="5"/>
+      <c r="G87" s="5" t="b" cm="1">
+        <f t="array" ref="G87">_xlfn._xlws.FILTER($P$54:$P$75, (ISBLANK($P$54:$P$75)=FALSE)*($M$54:$M$75=$C87)*($N$54:$N$75=$J87), "")</f>
+        <v>0</v>
+      </c>
+      <c r="H87" s="5" t="str" cm="1">
+        <f t="array" ref="H87">_xlfn._xlws.FILTER($Q$54:$Q$75, (ISBLANK($Q$54:$Q$75)=FALSE)*($M$54:$M$75=$C87)*($N$54:$N$75=$J87), "")</f>
+        <v>LootBoxGold</v>
+      </c>
+      <c r="I87" s="5" t="str" cm="1">
+        <f t="array" ref="I87">_xlfn._xlws.FILTER($R$54:$R$75, (ISBLANK($R$54:$R$75)=FALSE)*($M$54:$M$75=$C87)*($N$54:$N$75=$J87), "")</f>
+        <v/>
+      </c>
+      <c r="J87">
+        <f t="shared" si="12"/>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="88" spans="2:10" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="89" spans="2:10" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B89" s="8" t="str">
+        <f>_xlfn.CONCAT("stage",J89)</f>
+        <v>stage8</v>
+      </c>
+      <c r="C89" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="D89" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="E89" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="F89" s="5"/>
+      <c r="G89" s="5"/>
+      <c r="H89" s="5"/>
+      <c r="I89" s="5"/>
+      <c r="J89">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="90" spans="2:10" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B90" s="5"/>
+      <c r="C90" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="D90" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="E90" s="8" cm="1">
+        <f t="array" ref="E90">_xlfn.TAKE(_xlfn._xlws.FILTER($S$54:$S$75,$N$54:$N$75=J90, TRUE), 1)</f>
+        <v>550</v>
+      </c>
+      <c r="F90" s="5"/>
+      <c r="G90" s="5"/>
+      <c r="H90" s="5"/>
+      <c r="I90" s="5"/>
+      <c r="J90">
+        <f>J89</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="91" spans="2:10" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B91" s="5"/>
+      <c r="C91" s="8" t="s">
+        <v>180</v>
+      </c>
+      <c r="D91" s="5" t="str" cm="1">
+        <f t="array" ref="D91">_xlfn._xlws.FILTER($O$54:$O$75, ($M$54:$M$75=$C91)*($N$54:$N$75=$J91))</f>
+        <v>SeasonWheelTicketsReward</v>
+      </c>
+      <c r="E91" s="5"/>
+      <c r="F91" s="5"/>
+      <c r="G91" s="5" t="b" cm="1">
+        <f t="array" ref="G91">_xlfn._xlws.FILTER($P$54:$P$75, (ISBLANK($P$54:$P$75)=FALSE)*($M$54:$M$75=$C91)*($N$54:$N$75=$J91), "")</f>
+        <v>0</v>
+      </c>
+      <c r="H91" s="5" t="str" cm="1">
+        <f t="array" ref="H91">_xlfn._xlws.FILTER($Q$54:$Q$75, (ISBLANK($Q$54:$Q$75)=FALSE)*($M$54:$M$75=$C91)*($N$54:$N$75=$J91), "")</f>
+        <v>Basic</v>
+      </c>
+      <c r="I91" s="5" cm="1">
+        <f t="array" ref="I91">_xlfn._xlws.FILTER($R$54:$R$75, (ISBLANK($R$54:$R$75)=FALSE)*($M$54:$M$75=$C91)*($N$54:$N$75=$J91), "")</f>
+        <v>1</v>
+      </c>
+      <c r="J91">
+        <f t="shared" ref="J91:J92" si="13">J90</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="92" spans="2:10" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B92" s="5"/>
+      <c r="C92" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="D92" s="5" t="str" cm="1">
+        <f t="array" ref="D92">_xlfn._xlws.FILTER($O$54:$O$75, ($M$54:$M$75=$C92)*($N$54:$N$75=$J92))</f>
+        <v>SeasonCoreRandomBoosterReward</v>
+      </c>
+      <c r="E92" s="5"/>
+      <c r="F92" s="5"/>
+      <c r="G92" s="5" t="b" cm="1">
+        <f t="array" ref="G92">_xlfn._xlws.FILTER($P$54:$P$75, (ISBLANK($P$54:$P$75)=FALSE)*($M$54:$M$75=$C92)*($N$54:$N$75=$J92), "")</f>
+        <v>0</v>
+      </c>
+      <c r="H92" s="5" t="str" cm="1">
+        <f t="array" ref="H92">_xlfn._xlws.FILTER($Q$54:$Q$75, (ISBLANK($Q$54:$Q$75)=FALSE)*($M$54:$M$75=$C92)*($N$54:$N$75=$J92), "")</f>
+        <v>SeasonRandomBooster</v>
+      </c>
+      <c r="I92" s="5" cm="1">
+        <f t="array" ref="I92">_xlfn._xlws.FILTER($R$54:$R$75, (ISBLANK($R$54:$R$75)=FALSE)*($M$54:$M$75=$C92)*($N$54:$N$75=$J92), "")</f>
+        <v>5</v>
+      </c>
+      <c r="J92">
+        <f t="shared" si="13"/>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="93" spans="2:10" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="94" spans="2:10" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B94" s="8" t="str">
+        <f>_xlfn.CONCAT("stage",J94)</f>
+        <v>stage9</v>
+      </c>
+      <c r="C94" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="D94" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="E94" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="F94" s="5"/>
+      <c r="G94" s="5"/>
+      <c r="H94" s="5"/>
+      <c r="I94" s="5"/>
+      <c r="J94">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="95" spans="2:10" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B95" s="5"/>
+      <c r="C95" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="D95" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="E95" s="8" cm="1">
+        <f t="array" ref="E95">_xlfn.TAKE(_xlfn._xlws.FILTER($S$54:$S$75,$N$54:$N$75=J95, TRUE), 1)</f>
+        <v>600</v>
+      </c>
+      <c r="F95" s="5"/>
+      <c r="G95" s="5"/>
+      <c r="H95" s="5"/>
+      <c r="I95" s="5"/>
+      <c r="J95">
+        <f>J94</f>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="96" spans="2:10" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B96" s="5"/>
+      <c r="C96" s="8" t="s">
+        <v>180</v>
+      </c>
+      <c r="D96" s="5" t="str" cm="1">
+        <f t="array" ref="D96">_xlfn._xlws.FILTER($O$54:$O$75, ($M$54:$M$75=$C96)*($N$54:$N$75=$J96))</f>
+        <v>SeasonWheelTicketsReward</v>
+      </c>
+      <c r="E96" s="5"/>
+      <c r="F96" s="5"/>
+      <c r="G96" s="5" t="b" cm="1">
+        <f t="array" ref="G96">_xlfn._xlws.FILTER($P$54:$P$75, (ISBLANK($P$54:$P$75)=FALSE)*($M$54:$M$75=$C96)*($N$54:$N$75=$J96), "")</f>
+        <v>0</v>
+      </c>
+      <c r="H96" s="5" t="str" cm="1">
+        <f t="array" ref="H96">_xlfn._xlws.FILTER($Q$54:$Q$75, (ISBLANK($Q$54:$Q$75)=FALSE)*($M$54:$M$75=$C96)*($N$54:$N$75=$J96), "")</f>
+        <v>Basic</v>
+      </c>
+      <c r="I96" s="5" cm="1">
+        <f t="array" ref="I96">_xlfn._xlws.FILTER($R$54:$R$75, (ISBLANK($R$54:$R$75)=FALSE)*($M$54:$M$75=$C96)*($N$54:$N$75=$J96), "")</f>
+        <v>1</v>
+      </c>
+      <c r="J96">
+        <f t="shared" ref="J96:J97" si="14">J95</f>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="97" spans="2:10" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B97" s="5"/>
+      <c r="C97" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="D97" s="5" t="str" cm="1">
+        <f t="array" ref="D97">_xlfn._xlws.FILTER($O$54:$O$75, ($M$54:$M$75=$C97)*($N$54:$N$75=$J97))</f>
+        <v>SeasonLootBoxReward</v>
+      </c>
+      <c r="E97" s="5"/>
+      <c r="F97" s="5"/>
+      <c r="G97" s="5" t="b" cm="1">
+        <f t="array" ref="G97">_xlfn._xlws.FILTER($P$54:$P$75, (ISBLANK($P$54:$P$75)=FALSE)*($M$54:$M$75=$C97)*($N$54:$N$75=$J97), "")</f>
+        <v>0</v>
+      </c>
+      <c r="H97" s="5" t="str" cm="1">
+        <f t="array" ref="H97">_xlfn._xlws.FILTER($Q$54:$Q$75, (ISBLANK($Q$54:$Q$75)=FALSE)*($M$54:$M$75=$C97)*($N$54:$N$75=$J97), "")</f>
+        <v>LootBoxGold</v>
+      </c>
+      <c r="I97" s="5" t="str" cm="1">
+        <f t="array" ref="I97">_xlfn._xlws.FILTER($R$54:$R$75, (ISBLANK($R$54:$R$75)=FALSE)*($M$54:$M$75=$C97)*($N$54:$N$75=$J97), "")</f>
+        <v/>
+      </c>
+      <c r="J97">
+        <f t="shared" si="14"/>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="98" spans="2:10" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="99" spans="2:10" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B99" s="8" t="str">
+        <f>_xlfn.CONCAT("stage",J99)</f>
+        <v>stage10</v>
+      </c>
+      <c r="C99" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="D99" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="E99" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="F99" s="5"/>
+      <c r="G99" s="5"/>
+      <c r="H99" s="5"/>
+      <c r="I99" s="5"/>
+      <c r="J99">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="100" spans="2:10" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B100" s="5"/>
+      <c r="C100" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="D100" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="E100" s="8" cm="1">
+        <f t="array" ref="E100">_xlfn.TAKE(_xlfn._xlws.FILTER($S$54:$S$75,$N$54:$N$75=J100, TRUE), 1)</f>
+        <v>650</v>
+      </c>
+      <c r="F100" s="5"/>
+      <c r="G100" s="5"/>
+      <c r="H100" s="5"/>
+      <c r="I100" s="5"/>
+      <c r="J100">
+        <f>J99</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="101" spans="2:10" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B101" s="5"/>
+      <c r="C101" s="8" t="s">
+        <v>180</v>
+      </c>
+      <c r="D101" s="5" t="str" cm="1">
+        <f t="array" ref="D101">_xlfn._xlws.FILTER($O$54:$O$75, ($M$54:$M$75=$C101)*($N$54:$N$75=$J101))</f>
+        <v>SeasonCoreRandomBoosterReward</v>
+      </c>
+      <c r="E101" s="5"/>
+      <c r="F101" s="5"/>
+      <c r="G101" s="5" t="b" cm="1">
+        <f t="array" ref="G101">_xlfn._xlws.FILTER($P$54:$P$75, (ISBLANK($P$54:$P$75)=FALSE)*($M$54:$M$75=$C101)*($N$54:$N$75=$J101), "")</f>
+        <v>0</v>
+      </c>
+      <c r="H101" s="5" t="str" cm="1">
+        <f t="array" ref="H101">_xlfn._xlws.FILTER($Q$54:$Q$75, (ISBLANK($Q$54:$Q$75)=FALSE)*($M$54:$M$75=$C101)*($N$54:$N$75=$J101), "")</f>
+        <v>SeasonRandomBooster</v>
+      </c>
+      <c r="I101" s="5" cm="1">
+        <f t="array" ref="I101">_xlfn._xlws.FILTER($R$54:$R$75, (ISBLANK($R$54:$R$75)=FALSE)*($M$54:$M$75=$C101)*($N$54:$N$75=$J101), "")</f>
+        <v>3</v>
+      </c>
+      <c r="J101">
+        <f t="shared" ref="J101:J102" si="15">J100</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="102" spans="2:10" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B102" s="5"/>
+      <c r="C102" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="D102" s="5" t="str" cm="1">
+        <f t="array" ref="D102">_xlfn._xlws.FILTER($O$54:$O$75, ($M$54:$M$75=$C102)*($N$54:$N$75=$J102))</f>
+        <v>SeasonCoreRandomBoosterReward</v>
+      </c>
+      <c r="E102" s="5"/>
+      <c r="F102" s="5"/>
+      <c r="G102" s="5" t="b" cm="1">
+        <f t="array" ref="G102">_xlfn._xlws.FILTER($P$54:$P$75, (ISBLANK($P$54:$P$75)=FALSE)*($M$54:$M$75=$C102)*($N$54:$N$75=$J102), "")</f>
+        <v>1</v>
+      </c>
+      <c r="H102" s="5" t="str" cm="1">
+        <f t="array" ref="H102">_xlfn._xlws.FILTER($Q$54:$Q$75, (ISBLANK($Q$54:$Q$75)=FALSE)*($M$54:$M$75=$C102)*($N$54:$N$75=$J102), "")</f>
+        <v>SeasonRandomBooster</v>
+      </c>
+      <c r="I102" s="5" cm="1">
+        <f t="array" ref="I102">_xlfn._xlws.FILTER($R$54:$R$75, (ISBLANK($R$54:$R$75)=FALSE)*($M$54:$M$75=$C102)*($N$54:$N$75=$J102), "")</f>
+        <v>5</v>
+      </c>
+      <c r="J102">
+        <f t="shared" si="15"/>
+        <v>10</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="5">
+  <autoFilter ref="M53:W75" xr:uid="{90B4032F-FD98-457B-B53A-409A5704420A}"/>
+  <mergeCells count="19">
+    <mergeCell ref="B45:L45"/>
     <mergeCell ref="B5:L5"/>
     <mergeCell ref="B18:L18"/>
     <mergeCell ref="B19:L19"/>
     <mergeCell ref="B28:L28"/>
     <mergeCell ref="B7:L7"/>
+    <mergeCell ref="S74:S75"/>
+    <mergeCell ref="B47:I47"/>
+    <mergeCell ref="O52:R52"/>
+    <mergeCell ref="S54:S55"/>
+    <mergeCell ref="S56:S57"/>
+    <mergeCell ref="S58:S59"/>
+    <mergeCell ref="S60:S61"/>
+    <mergeCell ref="S62:S63"/>
+    <mergeCell ref="S64:S65"/>
+    <mergeCell ref="S66:S67"/>
+    <mergeCell ref="S68:S69"/>
+    <mergeCell ref="S70:S71"/>
+    <mergeCell ref="S72:S73"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>

</xml_diff>